<commit_message>
Added script to gather large dependencies
</commit_message>
<xml_diff>
--- a/tests/resources/workspace-001/sample-product-1.0.0/01_assets/example-001.xlsx
+++ b/tests/resources/workspace-001/sample-product-1.0.0/01_assets/example-001.xlsx
@@ -25,13 +25,292 @@
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="273" uniqueCount="168">
   <si>
+    <t>Canonical Name</t>
+  </si>
+  <si>
     <t>Id</t>
   </si>
   <si>
+    <t>SPDX Id</t>
+  </si>
+  <si>
+    <t>ScanCode Ids</t>
+  </si>
+  <si>
+    <t>RepresentedAs</t>
+  </si>
+  <si>
+    <t>OSI Status</t>
+  </si>
+  <si>
+    <t>Type Artifact</t>
+  </si>
+  <si>
+    <t>Type Web Module</t>
+  </si>
+  <si>
+    <t>BSD 3-Clause License</t>
+  </si>
+  <si>
+    <t>BSD-3-Clause</t>
+  </si>
+  <si>
+    <t>approved</t>
+  </si>
+  <si>
+    <t>x</t>
+  </si>
+  <si>
+    <t>BSD Zero Clause License</t>
+  </si>
+  <si>
+    <t>0BSD</t>
+  </si>
+  <si>
+    <t>Mozilla Public License 2.0</t>
+  </si>
+  <si>
+    <t>MPL-2.0</t>
+  </si>
+  <si>
+    <t>Apache License 2.0</t>
+  </si>
+  <si>
+    <t>Apache-2.0</t>
+  </si>
+  <si>
+    <t>MIT License</t>
+  </si>
+  <si>
+    <t>MIT</t>
+  </si>
+  <si>
+    <t>BSD alike</t>
+  </si>
+  <si>
+    <t>BSD-alike</t>
+  </si>
+  <si>
+    <t>Public Domain</t>
+  </si>
+  <si>
+    <t>Public-Domain</t>
+  </si>
+  <si>
+    <t>BSD 3-Clause License (copyright holder variant)</t>
+  </si>
+  <si>
+    <t>BSD-3-Clause-Copyright</t>
+  </si>
+  <si>
+    <t>Asset Id</t>
+  </si>
+  <si>
+    <t>Architecture</t>
+  </si>
+  <si>
+    <t>Asset Path</t>
+  </si>
+  <si>
+    <t>Checksum</t>
+  </si>
+  <si>
+    <t>Comment</t>
+  </si>
+  <si>
+    <t>Container Specified Licenses</t>
+  </si>
+  <si>
+    <t>Created</t>
+  </si>
+  <si>
+    <t>Digest</t>
+  </si>
+  <si>
+    <t>Image Id</t>
+  </si>
+  <si>
+    <t>Name</t>
+  </si>
+  <si>
+    <t>Organization URL</t>
+  </si>
+  <si>
+    <t>Os</t>
+  </si>
+  <si>
+    <t>Primary</t>
+  </si>
+  <si>
+    <t>Repository</t>
+  </si>
+  <si>
+    <t>Size</t>
+  </si>
+  <si>
+    <t>Type</t>
+  </si>
+  <si>
+    <t>URL</t>
+  </si>
+  <si>
+    <t>Version</t>
+  </si>
+  <si>
+    <t>config_architecture</t>
+  </si>
+  <si>
+    <t>config_build-date</t>
+  </si>
+  <si>
+    <t>config_description</t>
+  </si>
+  <si>
+    <t>config_distribution-scope</t>
+  </si>
+  <si>
+    <t>config_io.buildah.version</t>
+  </si>
+  <si>
+    <t>config_io.k8s.description</t>
+  </si>
+  <si>
+    <t>config_io.k8s.display-name</t>
+  </si>
+  <si>
+    <t>config_io.openshift.tags</t>
+  </si>
+  <si>
+    <t>config_maintainer</t>
+  </si>
+  <si>
+    <t>config_name</t>
+  </si>
+  <si>
+    <t>config_org.opencontainers.image.created</t>
+  </si>
+  <si>
+    <t>config_org.opencontainers.image.documentation</t>
+  </si>
+  <si>
+    <t>config_org.opencontainers.image.licenses</t>
+  </si>
+  <si>
+    <t>config_org.opencontainers.image.revision</t>
+  </si>
+  <si>
+    <t>config_org.opencontainers.image.source</t>
+  </si>
+  <si>
+    <t>config_org.opencontainers.image.title</t>
+  </si>
+  <si>
+    <t>config_org.opencontainers.image.url</t>
+  </si>
+  <si>
+    <t>config_org.opencontainers.image.version</t>
+  </si>
+  <si>
+    <t>config_summary</t>
+  </si>
+  <si>
+    <t>config_url</t>
+  </si>
+  <si>
+    <t>config_vcs-type</t>
+  </si>
+  <si>
+    <t>config_vendor</t>
+  </si>
+  <si>
+    <t>config_version</t>
+  </si>
+  <si>
+    <t>meta_LastTagTime</t>
+  </si>
+  <si>
     <t>CID-8ddfbf9408625337e69608156e0a075016b427b672d796cd694450222f88ac23</t>
   </si>
   <si>
-    <t>Checksum</t>
+    <t>x86_64</t>
+  </si>
+  <si>
+    <t>[keycloak-25.0.4.tar], keycloak-25.0.4.json, keycloak-25.0.4.tar</t>
+  </si>
+  <si>
+    <t>1fd2a6edd412dba4d243cabcc2cde1ac</t>
+  </si>
+  <si>
+    <t>buildkit.dockerfile.v0</t>
+  </si>
+  <si>
+    <t>2024-08-19T09:19:14</t>
+  </si>
+  <si>
+    <t>sha256:bf788a3b7fd737143f98d4cb514cb9599c896acee01a26b2117a10bd99e23e11</t>
+  </si>
+  <si>
+    <t>sha256:8ddfbf9408625337e69608156e0a075016b427b672d796cd694450222f88ac23</t>
+  </si>
+  <si>
+    <t>Keycloak Server Image</t>
+  </si>
+  <si>
+    <t>https://www.keycloak.org/</t>
+  </si>
+  <si>
+    <t>linux</t>
+  </si>
+  <si>
+    <t>keycloak/keycloak</t>
+  </si>
+  <si>
+    <t>432154175</t>
+  </si>
+  <si>
+    <t>container</t>
+  </si>
+  <si>
+    <t>25.0.4</t>
+  </si>
+  <si>
+    <t>2024-07-18T17:22:52</t>
+  </si>
+  <si>
+    <t>public</t>
+  </si>
+  <si>
+    <t>1.29.0</t>
+  </si>
+  <si>
+    <t>Keycloak Server</t>
+  </si>
+  <si>
+    <t>keycloak security identity</t>
+  </si>
+  <si>
+    <t>keycloak</t>
+  </si>
+  <si>
+    <t>2024-08-19T09:18:37.887Z</t>
+  </si>
+  <si>
+    <t>https://www.keycloak.org/documentation</t>
+  </si>
+  <si>
+    <t>52687e78792330893533b608b727af1ed8c69836</t>
+  </si>
+  <si>
+    <t>https://github.com/keycloak-rel/keycloak-rel</t>
+  </si>
+  <si>
+    <t>keycloak-rel</t>
+  </si>
+  <si>
+    <t>git</t>
+  </si>
+  <si>
+    <t>0001-01-01T00:00:00Z</t>
   </si>
   <si>
     <t>Component</t>
@@ -40,15 +319,9 @@
     <t>Group Id</t>
   </si>
   <si>
-    <t>Version</t>
-  </si>
-  <si>
     <t>Projects</t>
   </si>
   <si>
-    <t>Type</t>
-  </si>
-  <si>
     <t>Component Source Type</t>
   </si>
   <si>
@@ -197,210 +470,6 @@
   </si>
   <si>
     <t>b522a60d1f37b8f8b3b6ab58617df850b55fee6d82011b879a62574e068946aa</t>
-  </si>
-  <si>
-    <t>Asset Id</t>
-  </si>
-  <si>
-    <t>Architecture</t>
-  </si>
-  <si>
-    <t>Asset Path</t>
-  </si>
-  <si>
-    <t>Comment</t>
-  </si>
-  <si>
-    <t>Container Specified Licenses</t>
-  </si>
-  <si>
-    <t>Created</t>
-  </si>
-  <si>
-    <t>Digest</t>
-  </si>
-  <si>
-    <t>Image Id</t>
-  </si>
-  <si>
-    <t>Name</t>
-  </si>
-  <si>
-    <t>Organization URL</t>
-  </si>
-  <si>
-    <t>Os</t>
-  </si>
-  <si>
-    <t>Primary</t>
-  </si>
-  <si>
-    <t>Repository</t>
-  </si>
-  <si>
-    <t>Size</t>
-  </si>
-  <si>
-    <t>URL</t>
-  </si>
-  <si>
-    <t>config_architecture</t>
-  </si>
-  <si>
-    <t>config_build-date</t>
-  </si>
-  <si>
-    <t>config_description</t>
-  </si>
-  <si>
-    <t>config_distribution-scope</t>
-  </si>
-  <si>
-    <t>config_io.buildah.version</t>
-  </si>
-  <si>
-    <t>config_io.k8s.description</t>
-  </si>
-  <si>
-    <t>config_io.k8s.display-name</t>
-  </si>
-  <si>
-    <t>config_io.openshift.tags</t>
-  </si>
-  <si>
-    <t>config_maintainer</t>
-  </si>
-  <si>
-    <t>config_name</t>
-  </si>
-  <si>
-    <t>config_org.opencontainers.image.created</t>
-  </si>
-  <si>
-    <t>config_org.opencontainers.image.documentation</t>
-  </si>
-  <si>
-    <t>config_org.opencontainers.image.licenses</t>
-  </si>
-  <si>
-    <t>config_org.opencontainers.image.revision</t>
-  </si>
-  <si>
-    <t>config_org.opencontainers.image.source</t>
-  </si>
-  <si>
-    <t>config_org.opencontainers.image.title</t>
-  </si>
-  <si>
-    <t>config_org.opencontainers.image.url</t>
-  </si>
-  <si>
-    <t>config_org.opencontainers.image.version</t>
-  </si>
-  <si>
-    <t>config_summary</t>
-  </si>
-  <si>
-    <t>config_url</t>
-  </si>
-  <si>
-    <t>config_vcs-type</t>
-  </si>
-  <si>
-    <t>config_vendor</t>
-  </si>
-  <si>
-    <t>config_version</t>
-  </si>
-  <si>
-    <t>meta_LastTagTime</t>
-  </si>
-  <si>
-    <t>x86_64</t>
-  </si>
-  <si>
-    <t>[keycloak-25.0.4.tar], keycloak-25.0.4.json, keycloak-25.0.4.tar</t>
-  </si>
-  <si>
-    <t>1fd2a6edd412dba4d243cabcc2cde1ac</t>
-  </si>
-  <si>
-    <t>buildkit.dockerfile.v0</t>
-  </si>
-  <si>
-    <t>Apache-2.0</t>
-  </si>
-  <si>
-    <t>2024-08-19T09:19:14</t>
-  </si>
-  <si>
-    <t>sha256:bf788a3b7fd737143f98d4cb514cb9599c896acee01a26b2117a10bd99e23e11</t>
-  </si>
-  <si>
-    <t>sha256:8ddfbf9408625337e69608156e0a075016b427b672d796cd694450222f88ac23</t>
-  </si>
-  <si>
-    <t>Keycloak Server Image</t>
-  </si>
-  <si>
-    <t>https://www.keycloak.org/</t>
-  </si>
-  <si>
-    <t>linux</t>
-  </si>
-  <si>
-    <t>x</t>
-  </si>
-  <si>
-    <t>keycloak/keycloak</t>
-  </si>
-  <si>
-    <t>432154175</t>
-  </si>
-  <si>
-    <t>container</t>
-  </si>
-  <si>
-    <t>25.0.4</t>
-  </si>
-  <si>
-    <t>2024-07-18T17:22:52</t>
-  </si>
-  <si>
-    <t>public</t>
-  </si>
-  <si>
-    <t>1.29.0</t>
-  </si>
-  <si>
-    <t>Keycloak Server</t>
-  </si>
-  <si>
-    <t>keycloak security identity</t>
-  </si>
-  <si>
-    <t>keycloak</t>
-  </si>
-  <si>
-    <t>2024-08-19T09:18:37.887Z</t>
-  </si>
-  <si>
-    <t>https://www.keycloak.org/documentation</t>
-  </si>
-  <si>
-    <t>52687e78792330893533b608b727af1ed8c69836</t>
-  </si>
-  <si>
-    <t>https://github.com/keycloak-rel/keycloak-rel</t>
-  </si>
-  <si>
-    <t>keycloak-rel</t>
-  </si>
-  <si>
-    <t>git</t>
-  </si>
-  <si>
-    <t>0001-01-01T00:00:00Z</t>
   </si>
   <si>
     <t>License</t>
@@ -468,75 +537,6 @@
   </si>
   <si>
     <t>Vulnerability Assessment Dashboard</t>
-  </si>
-  <si>
-    <t>Canonical Name</t>
-  </si>
-  <si>
-    <t>SPDX Id</t>
-  </si>
-  <si>
-    <t>ScanCode Ids</t>
-  </si>
-  <si>
-    <t>RepresentedAs</t>
-  </si>
-  <si>
-    <t>OSI Status</t>
-  </si>
-  <si>
-    <t>Type Artifact</t>
-  </si>
-  <si>
-    <t>Type Web Module</t>
-  </si>
-  <si>
-    <t>BSD 3-Clause License</t>
-  </si>
-  <si>
-    <t>BSD-3-Clause</t>
-  </si>
-  <si>
-    <t>approved</t>
-  </si>
-  <si>
-    <t>BSD Zero Clause License</t>
-  </si>
-  <si>
-    <t>0BSD</t>
-  </si>
-  <si>
-    <t>Mozilla Public License 2.0</t>
-  </si>
-  <si>
-    <t>MPL-2.0</t>
-  </si>
-  <si>
-    <t>Apache License 2.0</t>
-  </si>
-  <si>
-    <t>MIT License</t>
-  </si>
-  <si>
-    <t>MIT</t>
-  </si>
-  <si>
-    <t>BSD alike</t>
-  </si>
-  <si>
-    <t>BSD-alike</t>
-  </si>
-  <si>
-    <t>Public Domain</t>
-  </si>
-  <si>
-    <t>Public-Domain</t>
-  </si>
-  <si>
-    <t>BSD 3-Clause License (copyright holder variant)</t>
-  </si>
-  <si>
-    <t>BSD-3-Clause-Copyright</t>
   </si>
 </sst>
 </file>
@@ -748,380 +748,380 @@
   <sheetData>
     <row r="1" customHeight="true" ht="170.0">
       <c r="A1" s="1" t="s">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B1" s="4" t="s">
-        <v>1</v>
+        <v>68</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>2</v>
+        <v>29</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>3</v>
+        <v>96</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>4</v>
+        <v>97</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>5</v>
+        <v>43</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>6</v>
+        <v>98</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>7</v>
+        <v>41</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>8</v>
+        <v>99</v>
       </c>
       <c r="J1" s="1" t="s">
-        <v>9</v>
+        <v>100</v>
       </c>
       <c r="K1" s="1" t="s">
-        <v>10</v>
+        <v>101</v>
       </c>
       <c r="L1" s="1" t="s">
-        <v>11</v>
+        <v>102</v>
       </c>
       <c r="M1" s="1" t="s">
-        <v>12</v>
+        <v>103</v>
       </c>
       <c r="N1" s="1" t="s">
-        <v>13</v>
+        <v>104</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>14</v>
+        <v>105</v>
       </c>
       <c r="B2" s="9" t="s">
-        <v>15</v>
+        <v>106</v>
       </c>
       <c r="C2" t="s">
-        <v>16</v>
+        <v>107</v>
       </c>
       <c r="D2" t="s">
-        <v>17</v>
+        <v>108</v>
       </c>
       <c r="E2" t="s">
-        <v>18</v>
+        <v>109</v>
       </c>
       <c r="F2" t="s">
-        <v>19</v>
+        <v>110</v>
       </c>
       <c r="G2" t="s">
-        <v>14</v>
+        <v>105</v>
       </c>
       <c r="H2" t="s">
-        <v>20</v>
+        <v>111</v>
       </c>
       <c r="I2" t="s">
-        <v>21</v>
+        <v>112</v>
       </c>
       <c r="J2" t="s">
-        <v>22</v>
+        <v>113</v>
       </c>
       <c r="K2" t="s">
-        <v>23</v>
+        <v>114</v>
       </c>
       <c r="L2" t="s">
-        <v>24</v>
+        <v>115</v>
       </c>
       <c r="M2" t="s">
-        <v>25</v>
+        <v>116</v>
       </c>
       <c r="N2" t="s">
-        <v>14</v>
+        <v>105</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>26</v>
+        <v>117</v>
       </c>
       <c r="B3" s="9" t="s">
-        <v>15</v>
+        <v>106</v>
       </c>
       <c r="C3" t="s">
-        <v>27</v>
+        <v>118</v>
       </c>
       <c r="D3" t="s">
-        <v>17</v>
+        <v>108</v>
       </c>
       <c r="E3" t="s">
-        <v>18</v>
+        <v>109</v>
       </c>
       <c r="F3" t="s">
-        <v>19</v>
+        <v>110</v>
       </c>
       <c r="G3" t="s">
-        <v>26</v>
+        <v>117</v>
       </c>
       <c r="H3" t="s">
-        <v>20</v>
+        <v>111</v>
       </c>
       <c r="I3" t="s">
-        <v>21</v>
+        <v>112</v>
       </c>
       <c r="J3" t="s">
-        <v>28</v>
+        <v>119</v>
       </c>
       <c r="K3" t="s">
-        <v>29</v>
+        <v>120</v>
       </c>
       <c r="L3" t="s">
-        <v>30</v>
+        <v>121</v>
       </c>
       <c r="M3" t="s">
-        <v>25</v>
+        <v>116</v>
       </c>
       <c r="N3" t="s">
-        <v>26</v>
+        <v>117</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>31</v>
+        <v>122</v>
       </c>
       <c r="B4" s="9" t="s">
-        <v>15</v>
+        <v>106</v>
       </c>
       <c r="C4" t="s">
-        <v>32</v>
+        <v>123</v>
       </c>
       <c r="D4" t="s">
-        <v>33</v>
+        <v>124</v>
       </c>
       <c r="E4" t="s">
-        <v>34</v>
+        <v>125</v>
       </c>
       <c r="F4" t="s">
-        <v>35</v>
+        <v>126</v>
       </c>
       <c r="G4" t="s">
-        <v>31</v>
+        <v>122</v>
       </c>
       <c r="H4" t="s">
-        <v>20</v>
+        <v>111</v>
       </c>
       <c r="I4" t="s">
-        <v>21</v>
+        <v>112</v>
       </c>
       <c r="J4" t="s">
-        <v>36</v>
+        <v>127</v>
       </c>
       <c r="K4" t="s">
-        <v>37</v>
+        <v>128</v>
       </c>
       <c r="M4" t="s">
-        <v>25</v>
+        <v>116</v>
       </c>
       <c r="N4" t="s">
-        <v>31</v>
+        <v>122</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>38</v>
+        <v>129</v>
       </c>
       <c r="B5" s="9" t="s">
-        <v>15</v>
+        <v>106</v>
       </c>
       <c r="C5" t="s">
-        <v>39</v>
+        <v>130</v>
       </c>
       <c r="D5" t="s">
-        <v>33</v>
+        <v>124</v>
       </c>
       <c r="E5" t="s">
-        <v>34</v>
+        <v>125</v>
       </c>
       <c r="F5" t="s">
-        <v>35</v>
+        <v>126</v>
       </c>
       <c r="G5" t="s">
-        <v>38</v>
+        <v>129</v>
       </c>
       <c r="H5" t="s">
-        <v>20</v>
+        <v>111</v>
       </c>
       <c r="I5" t="s">
-        <v>21</v>
+        <v>112</v>
       </c>
       <c r="J5" t="s">
-        <v>40</v>
+        <v>131</v>
       </c>
       <c r="K5" t="s">
-        <v>41</v>
+        <v>132</v>
       </c>
       <c r="M5" t="s">
-        <v>25</v>
+        <v>116</v>
       </c>
       <c r="N5" t="s">
-        <v>38</v>
+        <v>129</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="s">
-        <v>42</v>
+        <v>133</v>
       </c>
       <c r="B6" s="9" t="s">
-        <v>15</v>
+        <v>106</v>
       </c>
       <c r="C6" t="s">
-        <v>43</v>
+        <v>134</v>
       </c>
       <c r="D6" t="s">
-        <v>33</v>
+        <v>124</v>
       </c>
       <c r="E6" t="s">
-        <v>34</v>
+        <v>125</v>
       </c>
       <c r="F6" t="s">
-        <v>35</v>
+        <v>126</v>
       </c>
       <c r="G6" t="s">
-        <v>42</v>
+        <v>133</v>
       </c>
       <c r="H6" t="s">
-        <v>20</v>
+        <v>111</v>
       </c>
       <c r="I6" t="s">
-        <v>21</v>
+        <v>112</v>
       </c>
       <c r="J6" t="s">
-        <v>44</v>
+        <v>135</v>
       </c>
       <c r="K6" t="s">
-        <v>45</v>
+        <v>136</v>
       </c>
       <c r="M6" t="s">
-        <v>25</v>
+        <v>116</v>
       </c>
       <c r="N6" t="s">
-        <v>42</v>
+        <v>133</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="s">
-        <v>46</v>
+        <v>137</v>
       </c>
       <c r="B7" s="9" t="s">
-        <v>15</v>
+        <v>106</v>
       </c>
       <c r="C7" t="s">
-        <v>47</v>
+        <v>138</v>
       </c>
       <c r="D7" t="s">
-        <v>33</v>
+        <v>124</v>
       </c>
       <c r="E7" t="s">
-        <v>34</v>
+        <v>125</v>
       </c>
       <c r="F7" t="s">
-        <v>35</v>
+        <v>126</v>
       </c>
       <c r="G7" t="s">
-        <v>46</v>
+        <v>137</v>
       </c>
       <c r="H7" t="s">
-        <v>20</v>
+        <v>111</v>
       </c>
       <c r="I7" t="s">
-        <v>21</v>
+        <v>112</v>
       </c>
       <c r="J7" t="s">
-        <v>48</v>
+        <v>139</v>
       </c>
       <c r="K7" t="s">
-        <v>49</v>
+        <v>140</v>
       </c>
       <c r="M7" t="s">
-        <v>25</v>
+        <v>116</v>
       </c>
       <c r="N7" t="s">
-        <v>46</v>
+        <v>137</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="s">
-        <v>50</v>
+        <v>141</v>
       </c>
       <c r="B8" s="9" t="s">
-        <v>15</v>
+        <v>106</v>
       </c>
       <c r="C8" t="s">
-        <v>51</v>
+        <v>142</v>
       </c>
       <c r="D8" t="s">
-        <v>33</v>
+        <v>124</v>
       </c>
       <c r="E8" t="s">
-        <v>34</v>
+        <v>125</v>
       </c>
       <c r="F8" t="s">
-        <v>35</v>
+        <v>126</v>
       </c>
       <c r="G8" t="s">
-        <v>50</v>
+        <v>141</v>
       </c>
       <c r="H8" t="s">
-        <v>20</v>
+        <v>111</v>
       </c>
       <c r="I8" t="s">
-        <v>21</v>
+        <v>112</v>
       </c>
       <c r="J8" t="s">
-        <v>52</v>
+        <v>143</v>
       </c>
       <c r="K8" t="s">
-        <v>53</v>
+        <v>144</v>
       </c>
       <c r="M8" t="s">
-        <v>25</v>
+        <v>116</v>
       </c>
       <c r="N8" t="s">
-        <v>50</v>
+        <v>141</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="s">
-        <v>54</v>
+        <v>145</v>
       </c>
       <c r="B9" s="9" t="s">
-        <v>15</v>
+        <v>106</v>
       </c>
       <c r="C9" t="s">
-        <v>55</v>
+        <v>146</v>
       </c>
       <c r="D9" t="s">
-        <v>33</v>
+        <v>124</v>
       </c>
       <c r="E9" t="s">
-        <v>34</v>
+        <v>125</v>
       </c>
       <c r="F9" t="s">
-        <v>35</v>
+        <v>126</v>
       </c>
       <c r="G9" t="s">
-        <v>54</v>
+        <v>145</v>
       </c>
       <c r="H9" t="s">
-        <v>20</v>
+        <v>111</v>
       </c>
       <c r="I9" t="s">
-        <v>21</v>
+        <v>112</v>
       </c>
       <c r="J9" t="s">
-        <v>56</v>
+        <v>147</v>
       </c>
       <c r="K9" t="s">
-        <v>57</v>
+        <v>148</v>
       </c>
       <c r="M9" t="s">
-        <v>25</v>
+        <v>116</v>
       </c>
       <c r="N9" t="s">
-        <v>54</v>
+        <v>145</v>
       </c>
     </row>
   </sheetData>
@@ -1163,258 +1163,258 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="I1" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="J1" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="K1" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="L1" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="M1" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="N1" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="O1" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="P1" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="Q1" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="R1" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="S1" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="T1" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="U1" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="V1" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="W1" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="X1" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="Y1" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="Z1" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="AA1" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AB1" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AC1" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AD1" s="3" t="s">
+        <v>55</v>
+      </c>
+      <c r="AE1" s="3" t="s">
+        <v>56</v>
+      </c>
+      <c r="AF1" s="3" t="s">
+        <v>57</v>
+      </c>
+      <c r="AG1" s="3" t="s">
         <v>58</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="AH1" s="3" t="s">
         <v>59</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="AI1" s="3" t="s">
         <v>60</v>
       </c>
-      <c r="D1" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="E1" s="1" t="s">
+      <c r="AJ1" s="3" t="s">
         <v>61</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="AK1" s="3" t="s">
         <v>62</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="AL1" s="3" t="s">
         <v>63</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="AM1" s="3" t="s">
         <v>64</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="AN1" s="3" t="s">
         <v>65</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="AO1" s="3" t="s">
         <v>66</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="AP1" s="3" t="s">
         <v>67</v>
-      </c>
-      <c r="L1" s="1" t="s">
-        <v>68</v>
-      </c>
-      <c r="M1" s="1" t="s">
-        <v>69</v>
-      </c>
-      <c r="N1" s="1" t="s">
-        <v>70</v>
-      </c>
-      <c r="O1" s="1" t="s">
-        <v>71</v>
-      </c>
-      <c r="P1" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="Q1" s="1" t="s">
-        <v>72</v>
-      </c>
-      <c r="R1" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="S1" s="3" t="s">
-        <v>73</v>
-      </c>
-      <c r="T1" s="3" t="s">
-        <v>74</v>
-      </c>
-      <c r="U1" s="3" t="s">
-        <v>75</v>
-      </c>
-      <c r="V1" s="3" t="s">
-        <v>76</v>
-      </c>
-      <c r="W1" s="3" t="s">
-        <v>77</v>
-      </c>
-      <c r="X1" s="3" t="s">
-        <v>78</v>
-      </c>
-      <c r="Y1" s="3" t="s">
-        <v>79</v>
-      </c>
-      <c r="Z1" s="3" t="s">
-        <v>80</v>
-      </c>
-      <c r="AA1" s="3" t="s">
-        <v>81</v>
-      </c>
-      <c r="AB1" s="3" t="s">
-        <v>82</v>
-      </c>
-      <c r="AC1" s="3" t="s">
-        <v>83</v>
-      </c>
-      <c r="AD1" s="3" t="s">
-        <v>84</v>
-      </c>
-      <c r="AE1" s="3" t="s">
-        <v>85</v>
-      </c>
-      <c r="AF1" s="3" t="s">
-        <v>86</v>
-      </c>
-      <c r="AG1" s="3" t="s">
-        <v>87</v>
-      </c>
-      <c r="AH1" s="3" t="s">
-        <v>88</v>
-      </c>
-      <c r="AI1" s="3" t="s">
-        <v>89</v>
-      </c>
-      <c r="AJ1" s="3" t="s">
-        <v>90</v>
-      </c>
-      <c r="AK1" s="3" t="s">
-        <v>91</v>
-      </c>
-      <c r="AL1" s="3" t="s">
-        <v>92</v>
-      </c>
-      <c r="AM1" s="3" t="s">
-        <v>93</v>
-      </c>
-      <c r="AN1" s="3" t="s">
-        <v>94</v>
-      </c>
-      <c r="AO1" s="3" t="s">
-        <v>95</v>
-      </c>
-      <c r="AP1" s="3" t="s">
-        <v>96</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>1</v>
+        <v>68</v>
       </c>
       <c r="B2" t="s">
-        <v>97</v>
+        <v>69</v>
       </c>
       <c r="C2" t="s">
-        <v>98</v>
+        <v>70</v>
       </c>
       <c r="D2" t="s">
-        <v>99</v>
+        <v>71</v>
       </c>
       <c r="E2" t="s">
-        <v>100</v>
+        <v>72</v>
       </c>
       <c r="F2" t="s">
-        <v>101</v>
+        <v>17</v>
       </c>
       <c r="G2" t="s">
-        <v>102</v>
+        <v>73</v>
       </c>
       <c r="H2" t="s">
-        <v>103</v>
+        <v>74</v>
       </c>
       <c r="I2" t="s">
-        <v>104</v>
+        <v>75</v>
       </c>
       <c r="J2" t="s">
-        <v>105</v>
+        <v>76</v>
       </c>
       <c r="K2" t="s">
-        <v>106</v>
+        <v>77</v>
       </c>
       <c r="L2" t="s">
-        <v>107</v>
+        <v>78</v>
       </c>
       <c r="M2" t="s">
-        <v>108</v>
+        <v>11</v>
       </c>
       <c r="N2" t="s">
-        <v>109</v>
+        <v>79</v>
       </c>
       <c r="O2" t="s">
-        <v>110</v>
+        <v>80</v>
       </c>
       <c r="P2" t="s">
-        <v>111</v>
+        <v>81</v>
       </c>
       <c r="Q2" t="s">
-        <v>106</v>
+        <v>77</v>
       </c>
       <c r="R2" t="s">
-        <v>112</v>
+        <v>82</v>
       </c>
       <c r="S2" t="s">
-        <v>97</v>
+        <v>69</v>
       </c>
       <c r="T2" t="s">
-        <v>113</v>
+        <v>83</v>
       </c>
       <c r="U2" t="s">
-        <v>105</v>
+        <v>76</v>
       </c>
       <c r="V2" t="s">
-        <v>114</v>
+        <v>84</v>
       </c>
       <c r="W2" t="s">
-        <v>115</v>
+        <v>85</v>
       </c>
       <c r="X2" t="s">
-        <v>105</v>
+        <v>76</v>
       </c>
       <c r="Y2" t="s">
-        <v>116</v>
+        <v>86</v>
       </c>
       <c r="Z2" t="s">
-        <v>117</v>
+        <v>87</v>
       </c>
       <c r="AA2" t="s">
-        <v>106</v>
+        <v>77</v>
       </c>
       <c r="AB2" t="s">
-        <v>118</v>
+        <v>88</v>
       </c>
       <c r="AC2" t="s">
-        <v>119</v>
+        <v>89</v>
       </c>
       <c r="AD2" t="s">
-        <v>120</v>
+        <v>90</v>
       </c>
       <c r="AE2" t="s">
-        <v>101</v>
+        <v>17</v>
       </c>
       <c r="AF2" t="s">
-        <v>121</v>
+        <v>91</v>
       </c>
       <c r="AG2" t="s">
-        <v>122</v>
+        <v>92</v>
       </c>
       <c r="AH2" t="s">
-        <v>123</v>
+        <v>93</v>
       </c>
       <c r="AI2" t="s">
-        <v>122</v>
+        <v>92</v>
       </c>
       <c r="AJ2" t="s">
-        <v>112</v>
+        <v>82</v>
       </c>
       <c r="AK2" t="s">
-        <v>105</v>
+        <v>76</v>
       </c>
       <c r="AL2" t="s">
-        <v>106</v>
+        <v>77</v>
       </c>
       <c r="AM2" t="s">
-        <v>124</v>
+        <v>94</v>
       </c>
       <c r="AN2" t="s">
-        <v>106</v>
+        <v>77</v>
       </c>
       <c r="AO2" t="s">
-        <v>112</v>
+        <v>82</v>
       </c>
       <c r="AP2" t="s">
-        <v>125</v>
+        <v>95</v>
       </c>
     </row>
   </sheetData>
@@ -1430,42 +1430,42 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="s">
-        <v>3</v>
+        <v>96</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>5</v>
+        <v>43</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>126</v>
+        <v>149</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>127</v>
+        <v>150</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>128</v>
+        <v>151</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>129</v>
+        <v>152</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>61</v>
+        <v>30</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>33</v>
+        <v>124</v>
       </c>
       <c r="B2" t="s">
-        <v>35</v>
+        <v>126</v>
       </c>
       <c r="C2" t="s">
-        <v>130</v>
+        <v>153</v>
       </c>
       <c r="D2" t="s">
-        <v>131</v>
+        <v>154</v>
       </c>
       <c r="F2" t="s">
-        <v>132</v>
+        <v>155</v>
       </c>
     </row>
   </sheetData>
@@ -1481,149 +1481,149 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="s">
-        <v>145</v>
+        <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>146</v>
+        <v>2</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>147</v>
+        <v>3</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>148</v>
+        <v>4</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>149</v>
+        <v>5</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>150</v>
+        <v>6</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>151</v>
+        <v>7</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>152</v>
+        <v>8</v>
       </c>
       <c r="B2" t="s">
-        <v>153</v>
+        <v>9</v>
       </c>
       <c r="C2" t="s">
-        <v>153</v>
+        <v>9</v>
       </c>
       <c r="F2" t="s">
-        <v>154</v>
+        <v>10</v>
       </c>
       <c r="G2" t="s">
-        <v>108</v>
+        <v>11</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>155</v>
+        <v>12</v>
       </c>
       <c r="B3" t="s">
-        <v>156</v>
+        <v>13</v>
       </c>
       <c r="C3" t="s">
-        <v>156</v>
+        <v>13</v>
       </c>
       <c r="F3" t="s">
-        <v>154</v>
+        <v>10</v>
       </c>
       <c r="H3" t="s">
-        <v>108</v>
+        <v>11</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>157</v>
+        <v>14</v>
       </c>
       <c r="B4" t="s">
-        <v>158</v>
+        <v>15</v>
       </c>
       <c r="C4" t="s">
-        <v>158</v>
+        <v>15</v>
       </c>
       <c r="F4" t="s">
-        <v>154</v>
+        <v>10</v>
       </c>
       <c r="G4" t="s">
-        <v>108</v>
+        <v>11</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>159</v>
+        <v>16</v>
       </c>
       <c r="B5" t="s">
-        <v>101</v>
+        <v>17</v>
       </c>
       <c r="C5" t="s">
-        <v>101</v>
+        <v>17</v>
       </c>
       <c r="F5" t="s">
-        <v>154</v>
+        <v>10</v>
       </c>
       <c r="H5" t="s">
-        <v>108</v>
+        <v>11</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="s">
-        <v>160</v>
+        <v>18</v>
       </c>
       <c r="B6" t="s">
-        <v>161</v>
+        <v>19</v>
       </c>
       <c r="C6" t="s">
-        <v>161</v>
+        <v>19</v>
       </c>
       <c r="F6" t="s">
-        <v>154</v>
+        <v>10</v>
       </c>
       <c r="H6" t="s">
-        <v>108</v>
+        <v>11</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="s">
-        <v>162</v>
+        <v>20</v>
       </c>
       <c r="B7" t="s">
-        <v>163</v>
+        <v>21</v>
       </c>
       <c r="G7" t="s">
-        <v>108</v>
+        <v>11</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="s">
-        <v>164</v>
+        <v>22</v>
       </c>
       <c r="B8" t="s">
-        <v>165</v>
+        <v>23</v>
       </c>
       <c r="G8" t="s">
-        <v>108</v>
+        <v>11</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="s">
-        <v>166</v>
+        <v>24</v>
       </c>
       <c r="B9" t="s">
-        <v>167</v>
+        <v>25</v>
       </c>
       <c r="E9" t="s">
-        <v>152</v>
+        <v>8</v>
       </c>
       <c r="G9" t="s">
-        <v>108</v>
+        <v>11</v>
       </c>
     </row>
   </sheetData>
@@ -1639,48 +1639,48 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="s">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>133</v>
+        <v>156</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>134</v>
+        <v>157</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>135</v>
+        <v>158</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>136</v>
+        <v>159</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>137</v>
+        <v>160</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>138</v>
+        <v>161</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>139</v>
+        <v>162</v>
       </c>
       <c r="B2" t="s">
-        <v>140</v>
+        <v>163</v>
       </c>
       <c r="C2" t="s">
-        <v>141</v>
+        <v>164</v>
       </c>
       <c r="D2" t="s">
-        <v>142</v>
+        <v>165</v>
       </c>
       <c r="E2" t="s">
-        <v>142</v>
+        <v>165</v>
       </c>
       <c r="F2" t="s">
-        <v>143</v>
+        <v>166</v>
       </c>
       <c r="G2" t="s">
-        <v>144</v>
+        <v>167</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
added mirror auth test, added source aggregation test
</commit_message>
<xml_diff>
--- a/tests/resources/workspace-001/sample-product-1.0.0/01_assets/example-001.xlsx
+++ b/tests/resources/workspace-001/sample-product-1.0.0/01_assets/example-001.xlsx
@@ -25,243 +25,333 @@
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="273" uniqueCount="168">
   <si>
-    <t>Canonical Name</t>
-  </si>
-  <si>
     <t>Id</t>
   </si>
   <si>
-    <t>SPDX Id</t>
-  </si>
-  <si>
-    <t>ScanCode Ids</t>
-  </si>
-  <si>
-    <t>RepresentedAs</t>
-  </si>
-  <si>
-    <t>OSI Status</t>
-  </si>
-  <si>
-    <t>Type Artifact</t>
-  </si>
-  <si>
-    <t>Type Web Module</t>
-  </si>
-  <si>
-    <t>BSD 3-Clause License</t>
-  </si>
-  <si>
-    <t>BSD-3-Clause</t>
-  </si>
-  <si>
-    <t>approved</t>
+    <t>CID-8ddfbf9408625337e69608156e0a075016b427b672d796cd694450222f88ac23</t>
+  </si>
+  <si>
+    <t>Checksum</t>
+  </si>
+  <si>
+    <t>Component</t>
+  </si>
+  <si>
+    <t>Group Id</t>
+  </si>
+  <si>
+    <t>Version</t>
+  </si>
+  <si>
+    <t>Projects</t>
+  </si>
+  <si>
+    <t>Type</t>
+  </si>
+  <si>
+    <t>Component Source Type</t>
+  </si>
+  <si>
+    <t>Hash (SHA-1)</t>
+  </si>
+  <si>
+    <t>Hash (SHA-256)</t>
+  </si>
+  <si>
+    <t>PURL</t>
+  </si>
+  <si>
+    <t>Packaging</t>
+  </si>
+  <si>
+    <t>Path in Asset</t>
+  </si>
+  <si>
+    <t>log4j-api-2.14.0.jar</t>
+  </si>
+  <si>
+    <t>c</t>
+  </si>
+  <si>
+    <t>4876a0d414b3c2a01c10b6e96d70b62d</t>
+  </si>
+  <si>
+    <t>Apache Log4j</t>
+  </si>
+  <si>
+    <t>org.apache.logging.log4j</t>
+  </si>
+  <si>
+    <t>2.14.0</t>
+  </si>
+  <si>
+    <t>module</t>
+  </si>
+  <si>
+    <t>jar-module</t>
+  </si>
+  <si>
+    <t>23cdb2c6babad9b2b0dcf47c6a2c29d504e4c7a8</t>
+  </si>
+  <si>
+    <t>9791ac85aa3cdad633e512192766f84995eddf4db188cc42facec52a0dae15e8</t>
+  </si>
+  <si>
+    <t>pkg:maven/org.apache.logging.log4j/log4j-api@2.14.0?type=jar</t>
+  </si>
+  <si>
+    <t>jar</t>
+  </si>
+  <si>
+    <t>log4j-core-2.14.0.jar</t>
+  </si>
+  <si>
+    <t>862c00b2e854f9c0f1e8d8409d23d899</t>
+  </si>
+  <si>
+    <t>e257b0562453f73eabac1bc3181ba33e79d193ed</t>
+  </si>
+  <si>
+    <t>f04ee9c0ac417471d9127b5880b96c3147249f20674a8dbb88e9949d855382a8</t>
+  </si>
+  <si>
+    <t>pkg:maven/org.apache.logging.log4j/log4j-core@2.14.0?type=jar</t>
+  </si>
+  <si>
+    <t>spring-aop-5.3.14.jar</t>
+  </si>
+  <si>
+    <t>953a41d016a5bc9d9e8ace3d90d499c9</t>
+  </si>
+  <si>
+    <t>Spring Framework</t>
+  </si>
+  <si>
+    <t>org.springframework</t>
+  </si>
+  <si>
+    <t>5.3.14</t>
+  </si>
+  <si>
+    <t>f049146a55991e89c0f04b9624f1f69e1763d80f</t>
+  </si>
+  <si>
+    <t>1f6bb90bc78fa69506841c24c33f29790650e092dab96a35e56441f045ae216d</t>
+  </si>
+  <si>
+    <t>spring-beans-5.3.14.jar</t>
+  </si>
+  <si>
+    <t>04f9dc60a62319c97f140b8ebc98f797</t>
+  </si>
+  <si>
+    <t>24cc27af89edc1581a57bb15bc160d2353f40a0e</t>
+  </si>
+  <si>
+    <t>b354f54923139b8d86bc594452a6f53329da7b1e0c2a6402f9d9ca24837091ad</t>
+  </si>
+  <si>
+    <t>spring-context-5.3.14.jar</t>
+  </si>
+  <si>
+    <t>731eee1b78fa01375de10fd95b84455d</t>
+  </si>
+  <si>
+    <t>ce6042492f042131f602bdc83fcb412b142bdac5</t>
+  </si>
+  <si>
+    <t>25efd823c10f3afbe1b65efe97370def475d202dd91477f66eb5685e746e2819</t>
+  </si>
+  <si>
+    <t>spring-core-5.3.14.jar</t>
+  </si>
+  <si>
+    <t>b9d1f2454c4b7d94c058026d272dfc3c</t>
+  </si>
+  <si>
+    <t>d87ad19f9d8b9a3f1a143db5a2be34c61751aaa2</t>
+  </si>
+  <si>
+    <t>00ffcfb2671e0c8cab33f75939c97e04127fcfd2e0670032c59b6f48d791b772</t>
+  </si>
+  <si>
+    <t>spring-expression-5.3.14.jar</t>
+  </si>
+  <si>
+    <t>1d268dba90b89964d97254bae133a431</t>
+  </si>
+  <si>
+    <t>5cd4c568522b7084afac5d2ac6cb945b797b3f16</t>
+  </si>
+  <si>
+    <t>f196833d5bca28b12fbb4ae3265c0f0c4dc9fb4c726b3bfc4cabcc129cd21cf7</t>
+  </si>
+  <si>
+    <t>spring-jcl-5.3.14.jar</t>
+  </si>
+  <si>
+    <t>dd81ad7cd0aa5b6f0225d6a0341edd9a</t>
+  </si>
+  <si>
+    <t>ffcf745ed5ba32930771378316fd08e97986bec2</t>
+  </si>
+  <si>
+    <t>b522a60d1f37b8f8b3b6ab58617df850b55fee6d82011b879a62574e068946aa</t>
+  </si>
+  <si>
+    <t>Asset Id</t>
+  </si>
+  <si>
+    <t>Architecture</t>
+  </si>
+  <si>
+    <t>Asset Path</t>
+  </si>
+  <si>
+    <t>Comment</t>
+  </si>
+  <si>
+    <t>Container Specified Licenses</t>
+  </si>
+  <si>
+    <t>Created</t>
+  </si>
+  <si>
+    <t>Digest</t>
+  </si>
+  <si>
+    <t>Image Id</t>
+  </si>
+  <si>
+    <t>Name</t>
+  </si>
+  <si>
+    <t>Organization URL</t>
+  </si>
+  <si>
+    <t>Os</t>
+  </si>
+  <si>
+    <t>Primary</t>
+  </si>
+  <si>
+    <t>Repository</t>
+  </si>
+  <si>
+    <t>Size</t>
+  </si>
+  <si>
+    <t>URL</t>
+  </si>
+  <si>
+    <t>config_architecture</t>
+  </si>
+  <si>
+    <t>config_build-date</t>
+  </si>
+  <si>
+    <t>config_description</t>
+  </si>
+  <si>
+    <t>config_distribution-scope</t>
+  </si>
+  <si>
+    <t>config_io.buildah.version</t>
+  </si>
+  <si>
+    <t>config_io.k8s.description</t>
+  </si>
+  <si>
+    <t>config_io.k8s.display-name</t>
+  </si>
+  <si>
+    <t>config_io.openshift.tags</t>
+  </si>
+  <si>
+    <t>config_maintainer</t>
+  </si>
+  <si>
+    <t>config_name</t>
+  </si>
+  <si>
+    <t>config_org.opencontainers.image.created</t>
+  </si>
+  <si>
+    <t>config_org.opencontainers.image.documentation</t>
+  </si>
+  <si>
+    <t>config_org.opencontainers.image.licenses</t>
+  </si>
+  <si>
+    <t>config_org.opencontainers.image.revision</t>
+  </si>
+  <si>
+    <t>config_org.opencontainers.image.source</t>
+  </si>
+  <si>
+    <t>config_org.opencontainers.image.title</t>
+  </si>
+  <si>
+    <t>config_org.opencontainers.image.url</t>
+  </si>
+  <si>
+    <t>config_org.opencontainers.image.version</t>
+  </si>
+  <si>
+    <t>config_summary</t>
+  </si>
+  <si>
+    <t>config_url</t>
+  </si>
+  <si>
+    <t>config_vcs-type</t>
+  </si>
+  <si>
+    <t>config_vendor</t>
+  </si>
+  <si>
+    <t>config_version</t>
+  </si>
+  <si>
+    <t>meta_LastTagTime</t>
+  </si>
+  <si>
+    <t>x86_64</t>
+  </si>
+  <si>
+    <t>[keycloak-25.0.4.tar], keycloak-25.0.4.json, keycloak-25.0.4.tar</t>
+  </si>
+  <si>
+    <t>1fd2a6edd412dba4d243cabcc2cde1ac</t>
+  </si>
+  <si>
+    <t>buildkit.dockerfile.v0</t>
+  </si>
+  <si>
+    <t>Apache-2.0</t>
+  </si>
+  <si>
+    <t>2024-08-19T09:19:14</t>
+  </si>
+  <si>
+    <t>sha256:bf788a3b7fd737143f98d4cb514cb9599c896acee01a26b2117a10bd99e23e11</t>
+  </si>
+  <si>
+    <t>sha256:8ddfbf9408625337e69608156e0a075016b427b672d796cd694450222f88ac23</t>
+  </si>
+  <si>
+    <t>Keycloak Server Image</t>
+  </si>
+  <si>
+    <t>https://www.keycloak.org/</t>
+  </si>
+  <si>
+    <t>linux</t>
   </si>
   <si>
     <t>x</t>
   </si>
   <si>
-    <t>BSD Zero Clause License</t>
-  </si>
-  <si>
-    <t>0BSD</t>
-  </si>
-  <si>
-    <t>Mozilla Public License 2.0</t>
-  </si>
-  <si>
-    <t>MPL-2.0</t>
-  </si>
-  <si>
-    <t>Apache License 2.0</t>
-  </si>
-  <si>
-    <t>Apache-2.0</t>
-  </si>
-  <si>
-    <t>MIT License</t>
-  </si>
-  <si>
-    <t>MIT</t>
-  </si>
-  <si>
-    <t>BSD alike</t>
-  </si>
-  <si>
-    <t>BSD-alike</t>
-  </si>
-  <si>
-    <t>Public Domain</t>
-  </si>
-  <si>
-    <t>Public-Domain</t>
-  </si>
-  <si>
-    <t>BSD 3-Clause License (copyright holder variant)</t>
-  </si>
-  <si>
-    <t>BSD-3-Clause-Copyright</t>
-  </si>
-  <si>
-    <t>Asset Id</t>
-  </si>
-  <si>
-    <t>Architecture</t>
-  </si>
-  <si>
-    <t>Asset Path</t>
-  </si>
-  <si>
-    <t>Checksum</t>
-  </si>
-  <si>
-    <t>Comment</t>
-  </si>
-  <si>
-    <t>Container Specified Licenses</t>
-  </si>
-  <si>
-    <t>Created</t>
-  </si>
-  <si>
-    <t>Digest</t>
-  </si>
-  <si>
-    <t>Image Id</t>
-  </si>
-  <si>
-    <t>Name</t>
-  </si>
-  <si>
-    <t>Organization URL</t>
-  </si>
-  <si>
-    <t>Os</t>
-  </si>
-  <si>
-    <t>Primary</t>
-  </si>
-  <si>
-    <t>Repository</t>
-  </si>
-  <si>
-    <t>Size</t>
-  </si>
-  <si>
-    <t>Type</t>
-  </si>
-  <si>
-    <t>URL</t>
-  </si>
-  <si>
-    <t>Version</t>
-  </si>
-  <si>
-    <t>config_architecture</t>
-  </si>
-  <si>
-    <t>config_build-date</t>
-  </si>
-  <si>
-    <t>config_description</t>
-  </si>
-  <si>
-    <t>config_distribution-scope</t>
-  </si>
-  <si>
-    <t>config_io.buildah.version</t>
-  </si>
-  <si>
-    <t>config_io.k8s.description</t>
-  </si>
-  <si>
-    <t>config_io.k8s.display-name</t>
-  </si>
-  <si>
-    <t>config_io.openshift.tags</t>
-  </si>
-  <si>
-    <t>config_maintainer</t>
-  </si>
-  <si>
-    <t>config_name</t>
-  </si>
-  <si>
-    <t>config_org.opencontainers.image.created</t>
-  </si>
-  <si>
-    <t>config_org.opencontainers.image.documentation</t>
-  </si>
-  <si>
-    <t>config_org.opencontainers.image.licenses</t>
-  </si>
-  <si>
-    <t>config_org.opencontainers.image.revision</t>
-  </si>
-  <si>
-    <t>config_org.opencontainers.image.source</t>
-  </si>
-  <si>
-    <t>config_org.opencontainers.image.title</t>
-  </si>
-  <si>
-    <t>config_org.opencontainers.image.url</t>
-  </si>
-  <si>
-    <t>config_org.opencontainers.image.version</t>
-  </si>
-  <si>
-    <t>config_summary</t>
-  </si>
-  <si>
-    <t>config_url</t>
-  </si>
-  <si>
-    <t>config_vcs-type</t>
-  </si>
-  <si>
-    <t>config_vendor</t>
-  </si>
-  <si>
-    <t>config_version</t>
-  </si>
-  <si>
-    <t>meta_LastTagTime</t>
-  </si>
-  <si>
-    <t>CID-8ddfbf9408625337e69608156e0a075016b427b672d796cd694450222f88ac23</t>
-  </si>
-  <si>
-    <t>x86_64</t>
-  </si>
-  <si>
-    <t>[keycloak-25.0.4.tar], keycloak-25.0.4.json, keycloak-25.0.4.tar</t>
-  </si>
-  <si>
-    <t>1fd2a6edd412dba4d243cabcc2cde1ac</t>
-  </si>
-  <si>
-    <t>buildkit.dockerfile.v0</t>
-  </si>
-  <si>
-    <t>2024-08-19T09:19:14</t>
-  </si>
-  <si>
-    <t>sha256:bf788a3b7fd737143f98d4cb514cb9599c896acee01a26b2117a10bd99e23e11</t>
-  </si>
-  <si>
-    <t>sha256:8ddfbf9408625337e69608156e0a075016b427b672d796cd694450222f88ac23</t>
-  </si>
-  <si>
-    <t>Keycloak Server Image</t>
-  </si>
-  <si>
-    <t>https://www.keycloak.org/</t>
-  </si>
-  <si>
-    <t>linux</t>
-  </si>
-  <si>
     <t>keycloak/keycloak</t>
   </si>
   <si>
@@ -311,165 +401,6 @@
   </si>
   <si>
     <t>0001-01-01T00:00:00Z</t>
-  </si>
-  <si>
-    <t>Component</t>
-  </si>
-  <si>
-    <t>Group Id</t>
-  </si>
-  <si>
-    <t>Projects</t>
-  </si>
-  <si>
-    <t>Component Source Type</t>
-  </si>
-  <si>
-    <t>Hash (SHA-1)</t>
-  </si>
-  <si>
-    <t>Hash (SHA-256)</t>
-  </si>
-  <si>
-    <t>PURL</t>
-  </si>
-  <si>
-    <t>Packaging</t>
-  </si>
-  <si>
-    <t>Path in Asset</t>
-  </si>
-  <si>
-    <t>log4j-api-2.14.0.jar</t>
-  </si>
-  <si>
-    <t>c</t>
-  </si>
-  <si>
-    <t>4876a0d414b3c2a01c10b6e96d70b62d</t>
-  </si>
-  <si>
-    <t>Apache Log4j</t>
-  </si>
-  <si>
-    <t>org.apache.logging.log4j</t>
-  </si>
-  <si>
-    <t>2.14.0</t>
-  </si>
-  <si>
-    <t>module</t>
-  </si>
-  <si>
-    <t>jar-module</t>
-  </si>
-  <si>
-    <t>23cdb2c6babad9b2b0dcf47c6a2c29d504e4c7a8</t>
-  </si>
-  <si>
-    <t>9791ac85aa3cdad633e512192766f84995eddf4db188cc42facec52a0dae15e8</t>
-  </si>
-  <si>
-    <t>pkg:maven/org.apache.logging.log4j/log4j-api@2.14.0?type=jar</t>
-  </si>
-  <si>
-    <t>jar</t>
-  </si>
-  <si>
-    <t>log4j-core-2.14.0.jar</t>
-  </si>
-  <si>
-    <t>862c00b2e854f9c0f1e8d8409d23d899</t>
-  </si>
-  <si>
-    <t>e257b0562453f73eabac1bc3181ba33e79d193ed</t>
-  </si>
-  <si>
-    <t>f04ee9c0ac417471d9127b5880b96c3147249f20674a8dbb88e9949d855382a8</t>
-  </si>
-  <si>
-    <t>pkg:maven/org.apache.logging.log4j/log4j-core@2.14.0?type=jar</t>
-  </si>
-  <si>
-    <t>spring-aop-5.3.14.jar</t>
-  </si>
-  <si>
-    <t>953a41d016a5bc9d9e8ace3d90d499c9</t>
-  </si>
-  <si>
-    <t>Spring Framework</t>
-  </si>
-  <si>
-    <t>org.springframework</t>
-  </si>
-  <si>
-    <t>5.3.14</t>
-  </si>
-  <si>
-    <t>f049146a55991e89c0f04b9624f1f69e1763d80f</t>
-  </si>
-  <si>
-    <t>1f6bb90bc78fa69506841c24c33f29790650e092dab96a35e56441f045ae216d</t>
-  </si>
-  <si>
-    <t>spring-beans-5.3.14.jar</t>
-  </si>
-  <si>
-    <t>04f9dc60a62319c97f140b8ebc98f797</t>
-  </si>
-  <si>
-    <t>24cc27af89edc1581a57bb15bc160d2353f40a0e</t>
-  </si>
-  <si>
-    <t>b354f54923139b8d86bc594452a6f53329da7b1e0c2a6402f9d9ca24837091ad</t>
-  </si>
-  <si>
-    <t>spring-context-5.3.14.jar</t>
-  </si>
-  <si>
-    <t>731eee1b78fa01375de10fd95b84455d</t>
-  </si>
-  <si>
-    <t>ce6042492f042131f602bdc83fcb412b142bdac5</t>
-  </si>
-  <si>
-    <t>25efd823c10f3afbe1b65efe97370def475d202dd91477f66eb5685e746e2819</t>
-  </si>
-  <si>
-    <t>spring-core-5.3.14.jar</t>
-  </si>
-  <si>
-    <t>b9d1f2454c4b7d94c058026d272dfc3c</t>
-  </si>
-  <si>
-    <t>d87ad19f9d8b9a3f1a143db5a2be34c61751aaa2</t>
-  </si>
-  <si>
-    <t>00ffcfb2671e0c8cab33f75939c97e04127fcfd2e0670032c59b6f48d791b772</t>
-  </si>
-  <si>
-    <t>spring-expression-5.3.14.jar</t>
-  </si>
-  <si>
-    <t>1d268dba90b89964d97254bae133a431</t>
-  </si>
-  <si>
-    <t>5cd4c568522b7084afac5d2ac6cb945b797b3f16</t>
-  </si>
-  <si>
-    <t>f196833d5bca28b12fbb4ae3265c0f0c4dc9fb4c726b3bfc4cabcc129cd21cf7</t>
-  </si>
-  <si>
-    <t>spring-jcl-5.3.14.jar</t>
-  </si>
-  <si>
-    <t>dd81ad7cd0aa5b6f0225d6a0341edd9a</t>
-  </si>
-  <si>
-    <t>ffcf745ed5ba32930771378316fd08e97986bec2</t>
-  </si>
-  <si>
-    <t>b522a60d1f37b8f8b3b6ab58617df850b55fee6d82011b879a62574e068946aa</t>
   </si>
   <si>
     <t>License</t>
@@ -501,6 +432,75 @@
 &lt;p&gt;The subcomponent &lt;b&gt;CGLIB 3.3&lt;/b&gt; is licensed under the terms of the Apache License 2.0.&lt;/p&gt;
 &lt;p&gt;The subcomponent &lt;b&gt;Objenesis 3.1&lt;/b&gt; is licensed under the terms of the Apache License 2.0.&lt;/p&gt;
 &lt;p&gt;Per the NOTICE file in the Objenesis ZIP distribution downloaded from http://objenesis.org/download.html and corresponding to section 4d of the Apache License, Version 2.0, in this case for Objenesis:&lt;lq&gt;Objenesis Copyright 2006-2019 Joe Walnes, Henri Tremblay, Leonardo Mesquita&lt;/lq&gt;&lt;/p&gt;</t>
+  </si>
+  <si>
+    <t>Canonical Name</t>
+  </si>
+  <si>
+    <t>SPDX Id</t>
+  </si>
+  <si>
+    <t>ScanCode Ids</t>
+  </si>
+  <si>
+    <t>RepresentedAs</t>
+  </si>
+  <si>
+    <t>OSI Status</t>
+  </si>
+  <si>
+    <t>Type Artifact</t>
+  </si>
+  <si>
+    <t>Type Web Module</t>
+  </si>
+  <si>
+    <t>BSD 3-Clause License</t>
+  </si>
+  <si>
+    <t>BSD-3-Clause</t>
+  </si>
+  <si>
+    <t>approved</t>
+  </si>
+  <si>
+    <t>BSD Zero Clause License</t>
+  </si>
+  <si>
+    <t>0BSD</t>
+  </si>
+  <si>
+    <t>Mozilla Public License 2.0</t>
+  </si>
+  <si>
+    <t>MPL-2.0</t>
+  </si>
+  <si>
+    <t>Apache License 2.0</t>
+  </si>
+  <si>
+    <t>MIT License</t>
+  </si>
+  <si>
+    <t>MIT</t>
+  </si>
+  <si>
+    <t>BSD alike</t>
+  </si>
+  <si>
+    <t>BSD-alike</t>
+  </si>
+  <si>
+    <t>Public Domain</t>
+  </si>
+  <si>
+    <t>Public-Domain</t>
+  </si>
+  <si>
+    <t>BSD 3-Clause License (copyright holder variant)</t>
+  </si>
+  <si>
+    <t>BSD-3-Clause-Copyright</t>
   </si>
   <si>
     <t>Assessment-Context</t>
@@ -748,380 +748,380 @@
   <sheetData>
     <row r="1" customHeight="true" ht="170.0">
       <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="4" t="s">
         <v>1</v>
       </c>
-      <c r="B1" s="4" t="s">
-        <v>68</v>
-      </c>
       <c r="C1" s="1" t="s">
-        <v>29</v>
+        <v>2</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>96</v>
+        <v>3</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>97</v>
+        <v>4</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>43</v>
+        <v>5</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>98</v>
+        <v>6</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>41</v>
+        <v>7</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>99</v>
+        <v>8</v>
       </c>
       <c r="J1" s="1" t="s">
-        <v>100</v>
+        <v>9</v>
       </c>
       <c r="K1" s="1" t="s">
-        <v>101</v>
+        <v>10</v>
       </c>
       <c r="L1" s="1" t="s">
-        <v>102</v>
+        <v>11</v>
       </c>
       <c r="M1" s="1" t="s">
-        <v>103</v>
+        <v>12</v>
       </c>
       <c r="N1" s="1" t="s">
-        <v>104</v>
+        <v>13</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>105</v>
+        <v>14</v>
       </c>
       <c r="B2" s="9" t="s">
-        <v>106</v>
+        <v>15</v>
       </c>
       <c r="C2" t="s">
-        <v>107</v>
+        <v>16</v>
       </c>
       <c r="D2" t="s">
-        <v>108</v>
+        <v>17</v>
       </c>
       <c r="E2" t="s">
-        <v>109</v>
+        <v>18</v>
       </c>
       <c r="F2" t="s">
-        <v>110</v>
+        <v>19</v>
       </c>
       <c r="G2" t="s">
-        <v>105</v>
+        <v>14</v>
       </c>
       <c r="H2" t="s">
-        <v>111</v>
+        <v>20</v>
       </c>
       <c r="I2" t="s">
-        <v>112</v>
+        <v>21</v>
       </c>
       <c r="J2" t="s">
-        <v>113</v>
+        <v>22</v>
       </c>
       <c r="K2" t="s">
-        <v>114</v>
+        <v>23</v>
       </c>
       <c r="L2" t="s">
-        <v>115</v>
+        <v>24</v>
       </c>
       <c r="M2" t="s">
-        <v>116</v>
+        <v>25</v>
       </c>
       <c r="N2" t="s">
-        <v>105</v>
+        <v>14</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>117</v>
+        <v>26</v>
       </c>
       <c r="B3" s="9" t="s">
-        <v>106</v>
+        <v>15</v>
       </c>
       <c r="C3" t="s">
-        <v>118</v>
+        <v>27</v>
       </c>
       <c r="D3" t="s">
-        <v>108</v>
+        <v>17</v>
       </c>
       <c r="E3" t="s">
-        <v>109</v>
+        <v>18</v>
       </c>
       <c r="F3" t="s">
-        <v>110</v>
+        <v>19</v>
       </c>
       <c r="G3" t="s">
-        <v>117</v>
+        <v>26</v>
       </c>
       <c r="H3" t="s">
-        <v>111</v>
+        <v>20</v>
       </c>
       <c r="I3" t="s">
-        <v>112</v>
+        <v>21</v>
       </c>
       <c r="J3" t="s">
-        <v>119</v>
+        <v>28</v>
       </c>
       <c r="K3" t="s">
-        <v>120</v>
+        <v>29</v>
       </c>
       <c r="L3" t="s">
-        <v>121</v>
+        <v>30</v>
       </c>
       <c r="M3" t="s">
-        <v>116</v>
+        <v>25</v>
       </c>
       <c r="N3" t="s">
-        <v>117</v>
+        <v>26</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>122</v>
+        <v>31</v>
       </c>
       <c r="B4" s="9" t="s">
-        <v>106</v>
+        <v>15</v>
       </c>
       <c r="C4" t="s">
-        <v>123</v>
+        <v>32</v>
       </c>
       <c r="D4" t="s">
-        <v>124</v>
+        <v>33</v>
       </c>
       <c r="E4" t="s">
-        <v>125</v>
+        <v>34</v>
       </c>
       <c r="F4" t="s">
-        <v>126</v>
+        <v>35</v>
       </c>
       <c r="G4" t="s">
-        <v>122</v>
+        <v>31</v>
       </c>
       <c r="H4" t="s">
-        <v>111</v>
+        <v>20</v>
       </c>
       <c r="I4" t="s">
-        <v>112</v>
+        <v>21</v>
       </c>
       <c r="J4" t="s">
-        <v>127</v>
+        <v>36</v>
       </c>
       <c r="K4" t="s">
-        <v>128</v>
+        <v>37</v>
       </c>
       <c r="M4" t="s">
-        <v>116</v>
+        <v>25</v>
       </c>
       <c r="N4" t="s">
-        <v>122</v>
+        <v>31</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>129</v>
+        <v>38</v>
       </c>
       <c r="B5" s="9" t="s">
-        <v>106</v>
+        <v>15</v>
       </c>
       <c r="C5" t="s">
-        <v>130</v>
+        <v>39</v>
       </c>
       <c r="D5" t="s">
-        <v>124</v>
+        <v>33</v>
       </c>
       <c r="E5" t="s">
-        <v>125</v>
+        <v>34</v>
       </c>
       <c r="F5" t="s">
-        <v>126</v>
+        <v>35</v>
       </c>
       <c r="G5" t="s">
-        <v>129</v>
+        <v>38</v>
       </c>
       <c r="H5" t="s">
-        <v>111</v>
+        <v>20</v>
       </c>
       <c r="I5" t="s">
-        <v>112</v>
+        <v>21</v>
       </c>
       <c r="J5" t="s">
-        <v>131</v>
+        <v>40</v>
       </c>
       <c r="K5" t="s">
-        <v>132</v>
+        <v>41</v>
       </c>
       <c r="M5" t="s">
-        <v>116</v>
+        <v>25</v>
       </c>
       <c r="N5" t="s">
-        <v>129</v>
+        <v>38</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="s">
-        <v>133</v>
+        <v>42</v>
       </c>
       <c r="B6" s="9" t="s">
-        <v>106</v>
+        <v>15</v>
       </c>
       <c r="C6" t="s">
-        <v>134</v>
+        <v>43</v>
       </c>
       <c r="D6" t="s">
-        <v>124</v>
+        <v>33</v>
       </c>
       <c r="E6" t="s">
-        <v>125</v>
+        <v>34</v>
       </c>
       <c r="F6" t="s">
-        <v>126</v>
+        <v>35</v>
       </c>
       <c r="G6" t="s">
-        <v>133</v>
+        <v>42</v>
       </c>
       <c r="H6" t="s">
-        <v>111</v>
+        <v>20</v>
       </c>
       <c r="I6" t="s">
-        <v>112</v>
+        <v>21</v>
       </c>
       <c r="J6" t="s">
-        <v>135</v>
+        <v>44</v>
       </c>
       <c r="K6" t="s">
-        <v>136</v>
+        <v>45</v>
       </c>
       <c r="M6" t="s">
-        <v>116</v>
+        <v>25</v>
       </c>
       <c r="N6" t="s">
-        <v>133</v>
+        <v>42</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="s">
-        <v>137</v>
+        <v>46</v>
       </c>
       <c r="B7" s="9" t="s">
-        <v>106</v>
+        <v>15</v>
       </c>
       <c r="C7" t="s">
-        <v>138</v>
+        <v>47</v>
       </c>
       <c r="D7" t="s">
-        <v>124</v>
+        <v>33</v>
       </c>
       <c r="E7" t="s">
-        <v>125</v>
+        <v>34</v>
       </c>
       <c r="F7" t="s">
-        <v>126</v>
+        <v>35</v>
       </c>
       <c r="G7" t="s">
-        <v>137</v>
+        <v>46</v>
       </c>
       <c r="H7" t="s">
-        <v>111</v>
+        <v>20</v>
       </c>
       <c r="I7" t="s">
-        <v>112</v>
+        <v>21</v>
       </c>
       <c r="J7" t="s">
-        <v>139</v>
+        <v>48</v>
       </c>
       <c r="K7" t="s">
-        <v>140</v>
+        <v>49</v>
       </c>
       <c r="M7" t="s">
-        <v>116</v>
+        <v>25</v>
       </c>
       <c r="N7" t="s">
-        <v>137</v>
+        <v>46</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="s">
-        <v>141</v>
+        <v>50</v>
       </c>
       <c r="B8" s="9" t="s">
-        <v>106</v>
+        <v>15</v>
       </c>
       <c r="C8" t="s">
-        <v>142</v>
+        <v>51</v>
       </c>
       <c r="D8" t="s">
-        <v>124</v>
+        <v>33</v>
       </c>
       <c r="E8" t="s">
-        <v>125</v>
+        <v>34</v>
       </c>
       <c r="F8" t="s">
-        <v>126</v>
+        <v>35</v>
       </c>
       <c r="G8" t="s">
-        <v>141</v>
+        <v>50</v>
       </c>
       <c r="H8" t="s">
-        <v>111</v>
+        <v>20</v>
       </c>
       <c r="I8" t="s">
-        <v>112</v>
+        <v>21</v>
       </c>
       <c r="J8" t="s">
-        <v>143</v>
+        <v>52</v>
       </c>
       <c r="K8" t="s">
-        <v>144</v>
+        <v>53</v>
       </c>
       <c r="M8" t="s">
-        <v>116</v>
+        <v>25</v>
       </c>
       <c r="N8" t="s">
-        <v>141</v>
+        <v>50</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="s">
-        <v>145</v>
+        <v>54</v>
       </c>
       <c r="B9" s="9" t="s">
-        <v>106</v>
+        <v>15</v>
       </c>
       <c r="C9" t="s">
-        <v>146</v>
+        <v>55</v>
       </c>
       <c r="D9" t="s">
-        <v>124</v>
+        <v>33</v>
       </c>
       <c r="E9" t="s">
-        <v>125</v>
+        <v>34</v>
       </c>
       <c r="F9" t="s">
-        <v>126</v>
+        <v>35</v>
       </c>
       <c r="G9" t="s">
-        <v>145</v>
+        <v>54</v>
       </c>
       <c r="H9" t="s">
-        <v>111</v>
+        <v>20</v>
       </c>
       <c r="I9" t="s">
-        <v>112</v>
+        <v>21</v>
       </c>
       <c r="J9" t="s">
-        <v>147</v>
+        <v>56</v>
       </c>
       <c r="K9" t="s">
-        <v>148</v>
+        <v>57</v>
       </c>
       <c r="M9" t="s">
-        <v>116</v>
+        <v>25</v>
       </c>
       <c r="N9" t="s">
-        <v>145</v>
+        <v>54</v>
       </c>
     </row>
   </sheetData>
@@ -1163,258 +1163,258 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="s">
-        <v>26</v>
+        <v>58</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>27</v>
+        <v>59</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>28</v>
+        <v>60</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>29</v>
+        <v>2</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>30</v>
+        <v>61</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>31</v>
+        <v>62</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>32</v>
+        <v>63</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>33</v>
+        <v>64</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>34</v>
+        <v>65</v>
       </c>
       <c r="J1" s="1" t="s">
-        <v>35</v>
+        <v>66</v>
       </c>
       <c r="K1" s="1" t="s">
-        <v>36</v>
+        <v>67</v>
       </c>
       <c r="L1" s="1" t="s">
-        <v>37</v>
+        <v>68</v>
       </c>
       <c r="M1" s="1" t="s">
-        <v>38</v>
+        <v>69</v>
       </c>
       <c r="N1" s="1" t="s">
-        <v>39</v>
+        <v>70</v>
       </c>
       <c r="O1" s="1" t="s">
-        <v>40</v>
+        <v>71</v>
       </c>
       <c r="P1" s="1" t="s">
-        <v>41</v>
+        <v>7</v>
       </c>
       <c r="Q1" s="1" t="s">
-        <v>42</v>
+        <v>72</v>
       </c>
       <c r="R1" s="1" t="s">
-        <v>43</v>
+        <v>5</v>
       </c>
       <c r="S1" s="3" t="s">
-        <v>44</v>
+        <v>73</v>
       </c>
       <c r="T1" s="3" t="s">
-        <v>45</v>
+        <v>74</v>
       </c>
       <c r="U1" s="3" t="s">
-        <v>46</v>
+        <v>75</v>
       </c>
       <c r="V1" s="3" t="s">
-        <v>47</v>
+        <v>76</v>
       </c>
       <c r="W1" s="3" t="s">
-        <v>48</v>
+        <v>77</v>
       </c>
       <c r="X1" s="3" t="s">
-        <v>49</v>
+        <v>78</v>
       </c>
       <c r="Y1" s="3" t="s">
-        <v>50</v>
+        <v>79</v>
       </c>
       <c r="Z1" s="3" t="s">
-        <v>51</v>
+        <v>80</v>
       </c>
       <c r="AA1" s="3" t="s">
-        <v>52</v>
+        <v>81</v>
       </c>
       <c r="AB1" s="3" t="s">
-        <v>53</v>
+        <v>82</v>
       </c>
       <c r="AC1" s="3" t="s">
-        <v>54</v>
+        <v>83</v>
       </c>
       <c r="AD1" s="3" t="s">
-        <v>55</v>
+        <v>84</v>
       </c>
       <c r="AE1" s="3" t="s">
-        <v>56</v>
+        <v>85</v>
       </c>
       <c r="AF1" s="3" t="s">
-        <v>57</v>
+        <v>86</v>
       </c>
       <c r="AG1" s="3" t="s">
-        <v>58</v>
+        <v>87</v>
       </c>
       <c r="AH1" s="3" t="s">
-        <v>59</v>
+        <v>88</v>
       </c>
       <c r="AI1" s="3" t="s">
-        <v>60</v>
+        <v>89</v>
       </c>
       <c r="AJ1" s="3" t="s">
-        <v>61</v>
+        <v>90</v>
       </c>
       <c r="AK1" s="3" t="s">
-        <v>62</v>
+        <v>91</v>
       </c>
       <c r="AL1" s="3" t="s">
-        <v>63</v>
+        <v>92</v>
       </c>
       <c r="AM1" s="3" t="s">
-        <v>64</v>
+        <v>93</v>
       </c>
       <c r="AN1" s="3" t="s">
-        <v>65</v>
+        <v>94</v>
       </c>
       <c r="AO1" s="3" t="s">
-        <v>66</v>
+        <v>95</v>
       </c>
       <c r="AP1" s="3" t="s">
-        <v>67</v>
+        <v>96</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>68</v>
+        <v>1</v>
       </c>
       <c r="B2" t="s">
-        <v>69</v>
+        <v>97</v>
       </c>
       <c r="C2" t="s">
-        <v>70</v>
+        <v>98</v>
       </c>
       <c r="D2" t="s">
-        <v>71</v>
+        <v>99</v>
       </c>
       <c r="E2" t="s">
-        <v>72</v>
+        <v>100</v>
       </c>
       <c r="F2" t="s">
-        <v>17</v>
+        <v>101</v>
       </c>
       <c r="G2" t="s">
-        <v>73</v>
+        <v>102</v>
       </c>
       <c r="H2" t="s">
-        <v>74</v>
+        <v>103</v>
       </c>
       <c r="I2" t="s">
-        <v>75</v>
+        <v>104</v>
       </c>
       <c r="J2" t="s">
-        <v>76</v>
+        <v>105</v>
       </c>
       <c r="K2" t="s">
-        <v>77</v>
+        <v>106</v>
       </c>
       <c r="L2" t="s">
-        <v>78</v>
+        <v>107</v>
       </c>
       <c r="M2" t="s">
-        <v>11</v>
+        <v>108</v>
       </c>
       <c r="N2" t="s">
-        <v>79</v>
+        <v>109</v>
       </c>
       <c r="O2" t="s">
-        <v>80</v>
+        <v>110</v>
       </c>
       <c r="P2" t="s">
-        <v>81</v>
+        <v>111</v>
       </c>
       <c r="Q2" t="s">
-        <v>77</v>
+        <v>106</v>
       </c>
       <c r="R2" t="s">
-        <v>82</v>
+        <v>112</v>
       </c>
       <c r="S2" t="s">
-        <v>69</v>
+        <v>97</v>
       </c>
       <c r="T2" t="s">
-        <v>83</v>
+        <v>113</v>
       </c>
       <c r="U2" t="s">
-        <v>76</v>
+        <v>105</v>
       </c>
       <c r="V2" t="s">
-        <v>84</v>
+        <v>114</v>
       </c>
       <c r="W2" t="s">
-        <v>85</v>
+        <v>115</v>
       </c>
       <c r="X2" t="s">
-        <v>76</v>
+        <v>105</v>
       </c>
       <c r="Y2" t="s">
-        <v>86</v>
+        <v>116</v>
       </c>
       <c r="Z2" t="s">
-        <v>87</v>
+        <v>117</v>
       </c>
       <c r="AA2" t="s">
-        <v>77</v>
+        <v>106</v>
       </c>
       <c r="AB2" t="s">
-        <v>88</v>
+        <v>118</v>
       </c>
       <c r="AC2" t="s">
-        <v>89</v>
+        <v>119</v>
       </c>
       <c r="AD2" t="s">
-        <v>90</v>
+        <v>120</v>
       </c>
       <c r="AE2" t="s">
-        <v>17</v>
+        <v>101</v>
       </c>
       <c r="AF2" t="s">
-        <v>91</v>
+        <v>121</v>
       </c>
       <c r="AG2" t="s">
-        <v>92</v>
+        <v>122</v>
       </c>
       <c r="AH2" t="s">
-        <v>93</v>
+        <v>123</v>
       </c>
       <c r="AI2" t="s">
-        <v>92</v>
+        <v>122</v>
       </c>
       <c r="AJ2" t="s">
-        <v>82</v>
+        <v>112</v>
       </c>
       <c r="AK2" t="s">
-        <v>76</v>
+        <v>105</v>
       </c>
       <c r="AL2" t="s">
-        <v>77</v>
+        <v>106</v>
       </c>
       <c r="AM2" t="s">
-        <v>94</v>
+        <v>124</v>
       </c>
       <c r="AN2" t="s">
-        <v>77</v>
+        <v>106</v>
       </c>
       <c r="AO2" t="s">
-        <v>82</v>
+        <v>112</v>
       </c>
       <c r="AP2" t="s">
-        <v>95</v>
+        <v>125</v>
       </c>
     </row>
   </sheetData>
@@ -1430,42 +1430,42 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="s">
-        <v>96</v>
+        <v>3</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>43</v>
+        <v>5</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>149</v>
+        <v>126</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>150</v>
+        <v>127</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>151</v>
+        <v>128</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>152</v>
+        <v>129</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>30</v>
+        <v>61</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>124</v>
+        <v>33</v>
       </c>
       <c r="B2" t="s">
-        <v>126</v>
+        <v>35</v>
       </c>
       <c r="C2" t="s">
-        <v>153</v>
+        <v>130</v>
       </c>
       <c r="D2" t="s">
-        <v>154</v>
+        <v>131</v>
       </c>
       <c r="F2" t="s">
-        <v>155</v>
+        <v>132</v>
       </c>
     </row>
   </sheetData>
@@ -1481,149 +1481,149 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="s">
+        <v>133</v>
+      </c>
+      <c r="B1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
-        <v>1</v>
-      </c>
       <c r="C1" s="1" t="s">
-        <v>2</v>
+        <v>134</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>3</v>
+        <v>135</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>4</v>
+        <v>136</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>5</v>
+        <v>137</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>6</v>
+        <v>138</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>7</v>
+        <v>139</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>8</v>
+        <v>140</v>
       </c>
       <c r="B2" t="s">
-        <v>9</v>
+        <v>141</v>
       </c>
       <c r="C2" t="s">
-        <v>9</v>
+        <v>141</v>
       </c>
       <c r="F2" t="s">
-        <v>10</v>
+        <v>142</v>
       </c>
       <c r="G2" t="s">
-        <v>11</v>
+        <v>108</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>12</v>
+        <v>143</v>
       </c>
       <c r="B3" t="s">
-        <v>13</v>
+        <v>144</v>
       </c>
       <c r="C3" t="s">
-        <v>13</v>
+        <v>144</v>
       </c>
       <c r="F3" t="s">
-        <v>10</v>
+        <v>142</v>
       </c>
       <c r="H3" t="s">
-        <v>11</v>
+        <v>108</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>14</v>
+        <v>145</v>
       </c>
       <c r="B4" t="s">
-        <v>15</v>
+        <v>146</v>
       </c>
       <c r="C4" t="s">
-        <v>15</v>
+        <v>146</v>
       </c>
       <c r="F4" t="s">
-        <v>10</v>
+        <v>142</v>
       </c>
       <c r="G4" t="s">
-        <v>11</v>
+        <v>108</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>16</v>
+        <v>147</v>
       </c>
       <c r="B5" t="s">
-        <v>17</v>
+        <v>101</v>
       </c>
       <c r="C5" t="s">
-        <v>17</v>
+        <v>101</v>
       </c>
       <c r="F5" t="s">
-        <v>10</v>
+        <v>142</v>
       </c>
       <c r="H5" t="s">
-        <v>11</v>
+        <v>108</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="s">
-        <v>18</v>
+        <v>148</v>
       </c>
       <c r="B6" t="s">
-        <v>19</v>
+        <v>149</v>
       </c>
       <c r="C6" t="s">
-        <v>19</v>
+        <v>149</v>
       </c>
       <c r="F6" t="s">
-        <v>10</v>
+        <v>142</v>
       </c>
       <c r="H6" t="s">
-        <v>11</v>
+        <v>108</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="s">
-        <v>20</v>
+        <v>150</v>
       </c>
       <c r="B7" t="s">
-        <v>21</v>
+        <v>151</v>
       </c>
       <c r="G7" t="s">
-        <v>11</v>
+        <v>108</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="s">
-        <v>22</v>
+        <v>152</v>
       </c>
       <c r="B8" t="s">
-        <v>23</v>
+        <v>153</v>
       </c>
       <c r="G8" t="s">
-        <v>11</v>
+        <v>108</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="s">
-        <v>24</v>
+        <v>154</v>
       </c>
       <c r="B9" t="s">
-        <v>25</v>
+        <v>155</v>
       </c>
       <c r="E9" t="s">
-        <v>8</v>
+        <v>140</v>
       </c>
       <c r="G9" t="s">
-        <v>11</v>
+        <v>108</v>
       </c>
     </row>
   </sheetData>
@@ -1639,7 +1639,7 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="s">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>156</v>

</xml_diff>

<commit_message>
synced with experimental kontinuum branch
</commit_message>
<xml_diff>
--- a/tests/resources/workspace-001/sample-product-1.0.0/01_assets/example-001.xlsx
+++ b/tests/resources/workspace-001/sample-product-1.0.0/01_assets/example-001.xlsx
@@ -25,9 +25,84 @@
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="273" uniqueCount="168">
   <si>
+    <t>Canonical Name</t>
+  </si>
+  <si>
     <t>Id</t>
   </si>
   <si>
+    <t>SPDX Id</t>
+  </si>
+  <si>
+    <t>ScanCode Ids</t>
+  </si>
+  <si>
+    <t>RepresentedAs</t>
+  </si>
+  <si>
+    <t>OSI Status</t>
+  </si>
+  <si>
+    <t>Type Artifact</t>
+  </si>
+  <si>
+    <t>Type Web Module</t>
+  </si>
+  <si>
+    <t>BSD 3-Clause License</t>
+  </si>
+  <si>
+    <t>BSD-3-Clause</t>
+  </si>
+  <si>
+    <t>approved</t>
+  </si>
+  <si>
+    <t>x</t>
+  </si>
+  <si>
+    <t>BSD Zero Clause License</t>
+  </si>
+  <si>
+    <t>0BSD</t>
+  </si>
+  <si>
+    <t>Mozilla Public License 2.0</t>
+  </si>
+  <si>
+    <t>MPL-2.0</t>
+  </si>
+  <si>
+    <t>Apache License 2.0</t>
+  </si>
+  <si>
+    <t>Apache-2.0</t>
+  </si>
+  <si>
+    <t>MIT License</t>
+  </si>
+  <si>
+    <t>MIT</t>
+  </si>
+  <si>
+    <t>BSD alike</t>
+  </si>
+  <si>
+    <t>BSD-alike</t>
+  </si>
+  <si>
+    <t>Public Domain</t>
+  </si>
+  <si>
+    <t>Public-Domain</t>
+  </si>
+  <si>
+    <t>BSD 3-Clause License (copyright holder variant)</t>
+  </si>
+  <si>
+    <t>BSD-3-Clause-Copyright</t>
+  </si>
+  <si>
     <t>CID-8ddfbf9408625337e69608156e0a075016b427b672d796cd694450222f88ac23</t>
   </si>
   <si>
@@ -199,6 +274,42 @@
     <t>b522a60d1f37b8f8b3b6ab58617df850b55fee6d82011b879a62574e068946aa</t>
   </si>
   <si>
+    <t>Assessment-Context</t>
+  </si>
+  <si>
+    <t>Asset-Id</t>
+  </si>
+  <si>
+    <t>Footer</t>
+  </si>
+  <si>
+    <t>Subtitle</t>
+  </si>
+  <si>
+    <t>Tenant</t>
+  </si>
+  <si>
+    <t>Title</t>
+  </si>
+  <si>
+    <t>vad-customization</t>
+  </si>
+  <si>
+    <t>local</t>
+  </si>
+  <si>
+    <t>sample-product-1</t>
+  </si>
+  <si>
+    <t>advise_enrich-inventory</t>
+  </si>
+  <si>
+    <t>metaeffekt</t>
+  </si>
+  <si>
+    <t>Vulnerability Assessment Dashboard</t>
+  </si>
+  <si>
     <t>Asset Id</t>
   </si>
   <si>
@@ -328,9 +439,6 @@
     <t>buildkit.dockerfile.v0</t>
   </si>
   <si>
-    <t>Apache-2.0</t>
-  </si>
-  <si>
     <t>2024-08-19T09:19:14</t>
   </si>
   <si>
@@ -347,9 +455,6 @@
   </si>
   <si>
     <t>linux</t>
-  </si>
-  <si>
-    <t>x</t>
   </si>
   <si>
     <t>keycloak/keycloak</t>
@@ -432,111 +537,6 @@
 &lt;p&gt;The subcomponent &lt;b&gt;CGLIB 3.3&lt;/b&gt; is licensed under the terms of the Apache License 2.0.&lt;/p&gt;
 &lt;p&gt;The subcomponent &lt;b&gt;Objenesis 3.1&lt;/b&gt; is licensed under the terms of the Apache License 2.0.&lt;/p&gt;
 &lt;p&gt;Per the NOTICE file in the Objenesis ZIP distribution downloaded from http://objenesis.org/download.html and corresponding to section 4d of the Apache License, Version 2.0, in this case for Objenesis:&lt;lq&gt;Objenesis Copyright 2006-2019 Joe Walnes, Henri Tremblay, Leonardo Mesquita&lt;/lq&gt;&lt;/p&gt;</t>
-  </si>
-  <si>
-    <t>Canonical Name</t>
-  </si>
-  <si>
-    <t>SPDX Id</t>
-  </si>
-  <si>
-    <t>ScanCode Ids</t>
-  </si>
-  <si>
-    <t>RepresentedAs</t>
-  </si>
-  <si>
-    <t>OSI Status</t>
-  </si>
-  <si>
-    <t>Type Artifact</t>
-  </si>
-  <si>
-    <t>Type Web Module</t>
-  </si>
-  <si>
-    <t>BSD 3-Clause License</t>
-  </si>
-  <si>
-    <t>BSD-3-Clause</t>
-  </si>
-  <si>
-    <t>approved</t>
-  </si>
-  <si>
-    <t>BSD Zero Clause License</t>
-  </si>
-  <si>
-    <t>0BSD</t>
-  </si>
-  <si>
-    <t>Mozilla Public License 2.0</t>
-  </si>
-  <si>
-    <t>MPL-2.0</t>
-  </si>
-  <si>
-    <t>Apache License 2.0</t>
-  </si>
-  <si>
-    <t>MIT License</t>
-  </si>
-  <si>
-    <t>MIT</t>
-  </si>
-  <si>
-    <t>BSD alike</t>
-  </si>
-  <si>
-    <t>BSD-alike</t>
-  </si>
-  <si>
-    <t>Public Domain</t>
-  </si>
-  <si>
-    <t>Public-Domain</t>
-  </si>
-  <si>
-    <t>BSD 3-Clause License (copyright holder variant)</t>
-  </si>
-  <si>
-    <t>BSD-3-Clause-Copyright</t>
-  </si>
-  <si>
-    <t>Assessment-Context</t>
-  </si>
-  <si>
-    <t>Asset-Id</t>
-  </si>
-  <si>
-    <t>Footer</t>
-  </si>
-  <si>
-    <t>Subtitle</t>
-  </si>
-  <si>
-    <t>Tenant</t>
-  </si>
-  <si>
-    <t>Title</t>
-  </si>
-  <si>
-    <t>vad-customization</t>
-  </si>
-  <si>
-    <t>local</t>
-  </si>
-  <si>
-    <t>sample-product-1</t>
-  </si>
-  <si>
-    <t>advise_enrich-inventory</t>
-  </si>
-  <si>
-    <t>metaeffekt</t>
-  </si>
-  <si>
-    <t>Vulnerability Assessment Dashboard</t>
   </si>
 </sst>
 </file>
@@ -748,380 +748,380 @@
   <sheetData>
     <row r="1" customHeight="true" ht="170.0">
       <c r="A1" s="1" t="s">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B1" s="4" t="s">
-        <v>1</v>
+        <v>26</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>2</v>
+        <v>27</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>3</v>
+        <v>28</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>4</v>
+        <v>29</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>5</v>
+        <v>30</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>6</v>
+        <v>31</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>7</v>
+        <v>32</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>8</v>
+        <v>33</v>
       </c>
       <c r="J1" s="1" t="s">
-        <v>9</v>
+        <v>34</v>
       </c>
       <c r="K1" s="1" t="s">
-        <v>10</v>
+        <v>35</v>
       </c>
       <c r="L1" s="1" t="s">
-        <v>11</v>
+        <v>36</v>
       </c>
       <c r="M1" s="1" t="s">
-        <v>12</v>
+        <v>37</v>
       </c>
       <c r="N1" s="1" t="s">
-        <v>13</v>
+        <v>38</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>14</v>
+        <v>39</v>
       </c>
       <c r="B2" s="9" t="s">
-        <v>15</v>
+        <v>40</v>
       </c>
       <c r="C2" t="s">
-        <v>16</v>
+        <v>41</v>
       </c>
       <c r="D2" t="s">
-        <v>17</v>
+        <v>42</v>
       </c>
       <c r="E2" t="s">
-        <v>18</v>
+        <v>43</v>
       </c>
       <c r="F2" t="s">
-        <v>19</v>
+        <v>44</v>
       </c>
       <c r="G2" t="s">
-        <v>14</v>
+        <v>39</v>
       </c>
       <c r="H2" t="s">
-        <v>20</v>
+        <v>45</v>
       </c>
       <c r="I2" t="s">
-        <v>21</v>
+        <v>46</v>
       </c>
       <c r="J2" t="s">
-        <v>22</v>
+        <v>47</v>
       </c>
       <c r="K2" t="s">
-        <v>23</v>
+        <v>48</v>
       </c>
       <c r="L2" t="s">
-        <v>24</v>
+        <v>49</v>
       </c>
       <c r="M2" t="s">
-        <v>25</v>
+        <v>50</v>
       </c>
       <c r="N2" t="s">
-        <v>14</v>
+        <v>39</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>26</v>
+        <v>51</v>
       </c>
       <c r="B3" s="9" t="s">
-        <v>15</v>
+        <v>40</v>
       </c>
       <c r="C3" t="s">
-        <v>27</v>
+        <v>52</v>
       </c>
       <c r="D3" t="s">
-        <v>17</v>
+        <v>42</v>
       </c>
       <c r="E3" t="s">
-        <v>18</v>
+        <v>43</v>
       </c>
       <c r="F3" t="s">
-        <v>19</v>
+        <v>44</v>
       </c>
       <c r="G3" t="s">
-        <v>26</v>
+        <v>51</v>
       </c>
       <c r="H3" t="s">
-        <v>20</v>
+        <v>45</v>
       </c>
       <c r="I3" t="s">
-        <v>21</v>
+        <v>46</v>
       </c>
       <c r="J3" t="s">
-        <v>28</v>
+        <v>53</v>
       </c>
       <c r="K3" t="s">
-        <v>29</v>
+        <v>54</v>
       </c>
       <c r="L3" t="s">
-        <v>30</v>
+        <v>55</v>
       </c>
       <c r="M3" t="s">
-        <v>25</v>
+        <v>50</v>
       </c>
       <c r="N3" t="s">
-        <v>26</v>
+        <v>51</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>31</v>
+        <v>56</v>
       </c>
       <c r="B4" s="9" t="s">
-        <v>15</v>
+        <v>40</v>
       </c>
       <c r="C4" t="s">
-        <v>32</v>
+        <v>57</v>
       </c>
       <c r="D4" t="s">
-        <v>33</v>
+        <v>58</v>
       </c>
       <c r="E4" t="s">
-        <v>34</v>
+        <v>59</v>
       </c>
       <c r="F4" t="s">
-        <v>35</v>
+        <v>60</v>
       </c>
       <c r="G4" t="s">
-        <v>31</v>
+        <v>56</v>
       </c>
       <c r="H4" t="s">
-        <v>20</v>
+        <v>45</v>
       </c>
       <c r="I4" t="s">
-        <v>21</v>
+        <v>46</v>
       </c>
       <c r="J4" t="s">
-        <v>36</v>
+        <v>61</v>
       </c>
       <c r="K4" t="s">
-        <v>37</v>
+        <v>62</v>
       </c>
       <c r="M4" t="s">
-        <v>25</v>
+        <v>50</v>
       </c>
       <c r="N4" t="s">
-        <v>31</v>
+        <v>56</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>38</v>
+        <v>63</v>
       </c>
       <c r="B5" s="9" t="s">
-        <v>15</v>
+        <v>40</v>
       </c>
       <c r="C5" t="s">
-        <v>39</v>
+        <v>64</v>
       </c>
       <c r="D5" t="s">
-        <v>33</v>
+        <v>58</v>
       </c>
       <c r="E5" t="s">
-        <v>34</v>
+        <v>59</v>
       </c>
       <c r="F5" t="s">
-        <v>35</v>
+        <v>60</v>
       </c>
       <c r="G5" t="s">
-        <v>38</v>
+        <v>63</v>
       </c>
       <c r="H5" t="s">
-        <v>20</v>
+        <v>45</v>
       </c>
       <c r="I5" t="s">
-        <v>21</v>
+        <v>46</v>
       </c>
       <c r="J5" t="s">
-        <v>40</v>
+        <v>65</v>
       </c>
       <c r="K5" t="s">
-        <v>41</v>
+        <v>66</v>
       </c>
       <c r="M5" t="s">
-        <v>25</v>
+        <v>50</v>
       </c>
       <c r="N5" t="s">
-        <v>38</v>
+        <v>63</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="s">
-        <v>42</v>
+        <v>67</v>
       </c>
       <c r="B6" s="9" t="s">
-        <v>15</v>
+        <v>40</v>
       </c>
       <c r="C6" t="s">
-        <v>43</v>
+        <v>68</v>
       </c>
       <c r="D6" t="s">
-        <v>33</v>
+        <v>58</v>
       </c>
       <c r="E6" t="s">
-        <v>34</v>
+        <v>59</v>
       </c>
       <c r="F6" t="s">
-        <v>35</v>
+        <v>60</v>
       </c>
       <c r="G6" t="s">
-        <v>42</v>
+        <v>67</v>
       </c>
       <c r="H6" t="s">
-        <v>20</v>
+        <v>45</v>
       </c>
       <c r="I6" t="s">
-        <v>21</v>
+        <v>46</v>
       </c>
       <c r="J6" t="s">
-        <v>44</v>
+        <v>69</v>
       </c>
       <c r="K6" t="s">
-        <v>45</v>
+        <v>70</v>
       </c>
       <c r="M6" t="s">
-        <v>25</v>
+        <v>50</v>
       </c>
       <c r="N6" t="s">
-        <v>42</v>
+        <v>67</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="s">
+        <v>71</v>
+      </c>
+      <c r="B7" s="9" t="s">
+        <v>40</v>
+      </c>
+      <c r="C7" t="s">
+        <v>72</v>
+      </c>
+      <c r="D7" t="s">
+        <v>58</v>
+      </c>
+      <c r="E7" t="s">
+        <v>59</v>
+      </c>
+      <c r="F7" t="s">
+        <v>60</v>
+      </c>
+      <c r="G7" t="s">
+        <v>71</v>
+      </c>
+      <c r="H7" t="s">
+        <v>45</v>
+      </c>
+      <c r="I7" t="s">
         <v>46</v>
       </c>
-      <c r="B7" s="9" t="s">
-        <v>15</v>
-      </c>
-      <c r="C7" t="s">
-        <v>47</v>
-      </c>
-      <c r="D7" t="s">
-        <v>33</v>
-      </c>
-      <c r="E7" t="s">
-        <v>34</v>
-      </c>
-      <c r="F7" t="s">
-        <v>35</v>
-      </c>
-      <c r="G7" t="s">
-        <v>46</v>
-      </c>
-      <c r="H7" t="s">
-        <v>20</v>
-      </c>
-      <c r="I7" t="s">
-        <v>21</v>
-      </c>
       <c r="J7" t="s">
-        <v>48</v>
+        <v>73</v>
       </c>
       <c r="K7" t="s">
-        <v>49</v>
+        <v>74</v>
       </c>
       <c r="M7" t="s">
-        <v>25</v>
+        <v>50</v>
       </c>
       <c r="N7" t="s">
-        <v>46</v>
+        <v>71</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="s">
+        <v>75</v>
+      </c>
+      <c r="B8" s="9" t="s">
+        <v>40</v>
+      </c>
+      <c r="C8" t="s">
+        <v>76</v>
+      </c>
+      <c r="D8" t="s">
+        <v>58</v>
+      </c>
+      <c r="E8" t="s">
+        <v>59</v>
+      </c>
+      <c r="F8" t="s">
+        <v>60</v>
+      </c>
+      <c r="G8" t="s">
+        <v>75</v>
+      </c>
+      <c r="H8" t="s">
+        <v>45</v>
+      </c>
+      <c r="I8" t="s">
+        <v>46</v>
+      </c>
+      <c r="J8" t="s">
+        <v>77</v>
+      </c>
+      <c r="K8" t="s">
+        <v>78</v>
+      </c>
+      <c r="M8" t="s">
         <v>50</v>
       </c>
-      <c r="B8" s="9" t="s">
-        <v>15</v>
-      </c>
-      <c r="C8" t="s">
-        <v>51</v>
-      </c>
-      <c r="D8" t="s">
-        <v>33</v>
-      </c>
-      <c r="E8" t="s">
-        <v>34</v>
-      </c>
-      <c r="F8" t="s">
-        <v>35</v>
-      </c>
-      <c r="G8" t="s">
-        <v>50</v>
-      </c>
-      <c r="H8" t="s">
-        <v>20</v>
-      </c>
-      <c r="I8" t="s">
-        <v>21</v>
-      </c>
-      <c r="J8" t="s">
-        <v>52</v>
-      </c>
-      <c r="K8" t="s">
-        <v>53</v>
-      </c>
-      <c r="M8" t="s">
-        <v>25</v>
-      </c>
       <c r="N8" t="s">
-        <v>50</v>
+        <v>75</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="s">
-        <v>54</v>
+        <v>79</v>
       </c>
       <c r="B9" s="9" t="s">
-        <v>15</v>
+        <v>40</v>
       </c>
       <c r="C9" t="s">
-        <v>55</v>
+        <v>80</v>
       </c>
       <c r="D9" t="s">
-        <v>33</v>
+        <v>58</v>
       </c>
       <c r="E9" t="s">
-        <v>34</v>
+        <v>59</v>
       </c>
       <c r="F9" t="s">
-        <v>35</v>
+        <v>60</v>
       </c>
       <c r="G9" t="s">
-        <v>54</v>
+        <v>79</v>
       </c>
       <c r="H9" t="s">
-        <v>20</v>
+        <v>45</v>
       </c>
       <c r="I9" t="s">
-        <v>21</v>
+        <v>46</v>
       </c>
       <c r="J9" t="s">
-        <v>56</v>
+        <v>81</v>
       </c>
       <c r="K9" t="s">
-        <v>57</v>
+        <v>82</v>
       </c>
       <c r="M9" t="s">
-        <v>25</v>
+        <v>50</v>
       </c>
       <c r="N9" t="s">
-        <v>54</v>
+        <v>79</v>
       </c>
     </row>
   </sheetData>
@@ -1163,258 +1163,258 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="s">
-        <v>58</v>
+        <v>95</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>59</v>
+        <v>96</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>60</v>
+        <v>97</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>2</v>
+        <v>27</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>61</v>
+        <v>98</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>62</v>
+        <v>99</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>63</v>
+        <v>100</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>64</v>
+        <v>101</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>65</v>
+        <v>102</v>
       </c>
       <c r="J1" s="1" t="s">
-        <v>66</v>
+        <v>103</v>
       </c>
       <c r="K1" s="1" t="s">
-        <v>67</v>
+        <v>104</v>
       </c>
       <c r="L1" s="1" t="s">
-        <v>68</v>
+        <v>105</v>
       </c>
       <c r="M1" s="1" t="s">
-        <v>69</v>
+        <v>106</v>
       </c>
       <c r="N1" s="1" t="s">
-        <v>70</v>
+        <v>107</v>
       </c>
       <c r="O1" s="1" t="s">
-        <v>71</v>
+        <v>108</v>
       </c>
       <c r="P1" s="1" t="s">
-        <v>7</v>
+        <v>32</v>
       </c>
       <c r="Q1" s="1" t="s">
-        <v>72</v>
+        <v>109</v>
       </c>
       <c r="R1" s="1" t="s">
-        <v>5</v>
+        <v>30</v>
       </c>
       <c r="S1" s="3" t="s">
-        <v>73</v>
+        <v>110</v>
       </c>
       <c r="T1" s="3" t="s">
-        <v>74</v>
+        <v>111</v>
       </c>
       <c r="U1" s="3" t="s">
-        <v>75</v>
+        <v>112</v>
       </c>
       <c r="V1" s="3" t="s">
-        <v>76</v>
+        <v>113</v>
       </c>
       <c r="W1" s="3" t="s">
-        <v>77</v>
+        <v>114</v>
       </c>
       <c r="X1" s="3" t="s">
-        <v>78</v>
+        <v>115</v>
       </c>
       <c r="Y1" s="3" t="s">
-        <v>79</v>
+        <v>116</v>
       </c>
       <c r="Z1" s="3" t="s">
-        <v>80</v>
+        <v>117</v>
       </c>
       <c r="AA1" s="3" t="s">
-        <v>81</v>
+        <v>118</v>
       </c>
       <c r="AB1" s="3" t="s">
-        <v>82</v>
+        <v>119</v>
       </c>
       <c r="AC1" s="3" t="s">
-        <v>83</v>
+        <v>120</v>
       </c>
       <c r="AD1" s="3" t="s">
-        <v>84</v>
+        <v>121</v>
       </c>
       <c r="AE1" s="3" t="s">
-        <v>85</v>
+        <v>122</v>
       </c>
       <c r="AF1" s="3" t="s">
-        <v>86</v>
+        <v>123</v>
       </c>
       <c r="AG1" s="3" t="s">
-        <v>87</v>
+        <v>124</v>
       </c>
       <c r="AH1" s="3" t="s">
-        <v>88</v>
+        <v>125</v>
       </c>
       <c r="AI1" s="3" t="s">
-        <v>89</v>
+        <v>126</v>
       </c>
       <c r="AJ1" s="3" t="s">
-        <v>90</v>
+        <v>127</v>
       </c>
       <c r="AK1" s="3" t="s">
-        <v>91</v>
+        <v>128</v>
       </c>
       <c r="AL1" s="3" t="s">
-        <v>92</v>
+        <v>129</v>
       </c>
       <c r="AM1" s="3" t="s">
-        <v>93</v>
+        <v>130</v>
       </c>
       <c r="AN1" s="3" t="s">
-        <v>94</v>
+        <v>131</v>
       </c>
       <c r="AO1" s="3" t="s">
-        <v>95</v>
+        <v>132</v>
       </c>
       <c r="AP1" s="3" t="s">
-        <v>96</v>
+        <v>133</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>1</v>
+        <v>26</v>
       </c>
       <c r="B2" t="s">
-        <v>97</v>
+        <v>134</v>
       </c>
       <c r="C2" t="s">
-        <v>98</v>
+        <v>135</v>
       </c>
       <c r="D2" t="s">
-        <v>99</v>
+        <v>136</v>
       </c>
       <c r="E2" t="s">
-        <v>100</v>
+        <v>137</v>
       </c>
       <c r="F2" t="s">
-        <v>101</v>
+        <v>17</v>
       </c>
       <c r="G2" t="s">
-        <v>102</v>
+        <v>138</v>
       </c>
       <c r="H2" t="s">
-        <v>103</v>
+        <v>139</v>
       </c>
       <c r="I2" t="s">
-        <v>104</v>
+        <v>140</v>
       </c>
       <c r="J2" t="s">
-        <v>105</v>
+        <v>141</v>
       </c>
       <c r="K2" t="s">
-        <v>106</v>
+        <v>142</v>
       </c>
       <c r="L2" t="s">
-        <v>107</v>
+        <v>143</v>
       </c>
       <c r="M2" t="s">
-        <v>108</v>
+        <v>11</v>
       </c>
       <c r="N2" t="s">
-        <v>109</v>
+        <v>144</v>
       </c>
       <c r="O2" t="s">
-        <v>110</v>
+        <v>145</v>
       </c>
       <c r="P2" t="s">
-        <v>111</v>
+        <v>146</v>
       </c>
       <c r="Q2" t="s">
-        <v>106</v>
+        <v>142</v>
       </c>
       <c r="R2" t="s">
-        <v>112</v>
+        <v>147</v>
       </c>
       <c r="S2" t="s">
-        <v>97</v>
+        <v>134</v>
       </c>
       <c r="T2" t="s">
-        <v>113</v>
+        <v>148</v>
       </c>
       <c r="U2" t="s">
-        <v>105</v>
+        <v>141</v>
       </c>
       <c r="V2" t="s">
-        <v>114</v>
+        <v>149</v>
       </c>
       <c r="W2" t="s">
-        <v>115</v>
+        <v>150</v>
       </c>
       <c r="X2" t="s">
-        <v>105</v>
+        <v>141</v>
       </c>
       <c r="Y2" t="s">
-        <v>116</v>
+        <v>151</v>
       </c>
       <c r="Z2" t="s">
-        <v>117</v>
+        <v>152</v>
       </c>
       <c r="AA2" t="s">
-        <v>106</v>
+        <v>142</v>
       </c>
       <c r="AB2" t="s">
-        <v>118</v>
+        <v>153</v>
       </c>
       <c r="AC2" t="s">
-        <v>119</v>
+        <v>154</v>
       </c>
       <c r="AD2" t="s">
-        <v>120</v>
+        <v>155</v>
       </c>
       <c r="AE2" t="s">
-        <v>101</v>
+        <v>17</v>
       </c>
       <c r="AF2" t="s">
-        <v>121</v>
+        <v>156</v>
       </c>
       <c r="AG2" t="s">
-        <v>122</v>
+        <v>157</v>
       </c>
       <c r="AH2" t="s">
-        <v>123</v>
+        <v>158</v>
       </c>
       <c r="AI2" t="s">
-        <v>122</v>
+        <v>157</v>
       </c>
       <c r="AJ2" t="s">
-        <v>112</v>
+        <v>147</v>
       </c>
       <c r="AK2" t="s">
-        <v>105</v>
+        <v>141</v>
       </c>
       <c r="AL2" t="s">
-        <v>106</v>
+        <v>142</v>
       </c>
       <c r="AM2" t="s">
-        <v>124</v>
+        <v>159</v>
       </c>
       <c r="AN2" t="s">
-        <v>106</v>
+        <v>142</v>
       </c>
       <c r="AO2" t="s">
-        <v>112</v>
+        <v>147</v>
       </c>
       <c r="AP2" t="s">
-        <v>125</v>
+        <v>160</v>
       </c>
     </row>
   </sheetData>
@@ -1430,42 +1430,42 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="s">
-        <v>3</v>
+        <v>28</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>5</v>
+        <v>30</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>126</v>
+        <v>161</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>127</v>
+        <v>162</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>128</v>
+        <v>163</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>129</v>
+        <v>164</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>61</v>
+        <v>98</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>33</v>
+        <v>58</v>
       </c>
       <c r="B2" t="s">
-        <v>35</v>
+        <v>60</v>
       </c>
       <c r="C2" t="s">
-        <v>130</v>
+        <v>165</v>
       </c>
       <c r="D2" t="s">
-        <v>131</v>
+        <v>166</v>
       </c>
       <c r="F2" t="s">
-        <v>132</v>
+        <v>167</v>
       </c>
     </row>
   </sheetData>
@@ -1481,149 +1481,149 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="s">
-        <v>133</v>
+        <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>134</v>
+        <v>2</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>135</v>
+        <v>3</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>136</v>
+        <v>4</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>137</v>
+        <v>5</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>138</v>
+        <v>6</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>139</v>
+        <v>7</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>140</v>
+        <v>8</v>
       </c>
       <c r="B2" t="s">
-        <v>141</v>
+        <v>9</v>
       </c>
       <c r="C2" t="s">
-        <v>141</v>
+        <v>9</v>
       </c>
       <c r="F2" t="s">
-        <v>142</v>
+        <v>10</v>
       </c>
       <c r="G2" t="s">
-        <v>108</v>
+        <v>11</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>143</v>
+        <v>12</v>
       </c>
       <c r="B3" t="s">
-        <v>144</v>
+        <v>13</v>
       </c>
       <c r="C3" t="s">
-        <v>144</v>
+        <v>13</v>
       </c>
       <c r="F3" t="s">
-        <v>142</v>
+        <v>10</v>
       </c>
       <c r="H3" t="s">
-        <v>108</v>
+        <v>11</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>145</v>
+        <v>14</v>
       </c>
       <c r="B4" t="s">
-        <v>146</v>
+        <v>15</v>
       </c>
       <c r="C4" t="s">
-        <v>146</v>
+        <v>15</v>
       </c>
       <c r="F4" t="s">
-        <v>142</v>
+        <v>10</v>
       </c>
       <c r="G4" t="s">
-        <v>108</v>
+        <v>11</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>147</v>
+        <v>16</v>
       </c>
       <c r="B5" t="s">
-        <v>101</v>
+        <v>17</v>
       </c>
       <c r="C5" t="s">
-        <v>101</v>
+        <v>17</v>
       </c>
       <c r="F5" t="s">
-        <v>142</v>
+        <v>10</v>
       </c>
       <c r="H5" t="s">
-        <v>108</v>
+        <v>11</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="s">
-        <v>148</v>
+        <v>18</v>
       </c>
       <c r="B6" t="s">
-        <v>149</v>
+        <v>19</v>
       </c>
       <c r="C6" t="s">
-        <v>149</v>
+        <v>19</v>
       </c>
       <c r="F6" t="s">
-        <v>142</v>
+        <v>10</v>
       </c>
       <c r="H6" t="s">
-        <v>108</v>
+        <v>11</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="s">
-        <v>150</v>
+        <v>20</v>
       </c>
       <c r="B7" t="s">
-        <v>151</v>
+        <v>21</v>
       </c>
       <c r="G7" t="s">
-        <v>108</v>
+        <v>11</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="s">
-        <v>152</v>
+        <v>22</v>
       </c>
       <c r="B8" t="s">
-        <v>153</v>
+        <v>23</v>
       </c>
       <c r="G8" t="s">
-        <v>108</v>
+        <v>11</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="s">
-        <v>154</v>
+        <v>24</v>
       </c>
       <c r="B9" t="s">
-        <v>155</v>
+        <v>25</v>
       </c>
       <c r="E9" t="s">
-        <v>140</v>
+        <v>8</v>
       </c>
       <c r="G9" t="s">
-        <v>108</v>
+        <v>11</v>
       </c>
     </row>
   </sheetData>
@@ -1639,48 +1639,48 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="s">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>156</v>
+        <v>83</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>157</v>
+        <v>84</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>158</v>
+        <v>85</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>159</v>
+        <v>86</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>160</v>
+        <v>87</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>161</v>
+        <v>88</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>162</v>
+        <v>89</v>
       </c>
       <c r="B2" t="s">
-        <v>163</v>
+        <v>90</v>
       </c>
       <c r="C2" t="s">
-        <v>164</v>
+        <v>91</v>
       </c>
       <c r="D2" t="s">
-        <v>165</v>
+        <v>92</v>
       </c>
       <c r="E2" t="s">
-        <v>165</v>
+        <v>92</v>
       </c>
       <c r="F2" t="s">
-        <v>166</v>
+        <v>93</v>
       </c>
       <c r="G2" t="s">
-        <v>167</v>
+        <v>94</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
fixed execute kotlin script
</commit_message>
<xml_diff>
--- a/tests/resources/workspace-001/sample-product-1.0.0/01_assets/example-001.xlsx
+++ b/tests/resources/workspace-001/sample-product-1.0.0/01_assets/example-001.xlsx
@@ -103,12 +103,213 @@
     <t>BSD-3-Clause-Copyright</t>
   </si>
   <si>
+    <t>Assessment-Context</t>
+  </si>
+  <si>
+    <t>Asset-Id</t>
+  </si>
+  <si>
+    <t>Footer</t>
+  </si>
+  <si>
+    <t>Subtitle</t>
+  </si>
+  <si>
+    <t>Tenant</t>
+  </si>
+  <si>
+    <t>Title</t>
+  </si>
+  <si>
+    <t>vad-customization</t>
+  </si>
+  <si>
+    <t>local</t>
+  </si>
+  <si>
+    <t>sample-product-1</t>
+  </si>
+  <si>
+    <t>advise_enrich-inventory</t>
+  </si>
+  <si>
+    <t>metaeffekt</t>
+  </si>
+  <si>
+    <t>Vulnerability Assessment Dashboard</t>
+  </si>
+  <si>
+    <t>CID-8ddfbf9408625337e69608156e0a075016b427b672d796cd694450222f88ac23</t>
+  </si>
+  <si>
+    <t>Checksum</t>
+  </si>
+  <si>
     <t>Component</t>
   </si>
   <si>
+    <t>Group Id</t>
+  </si>
+  <si>
     <t>Version</t>
   </si>
   <si>
+    <t>Projects</t>
+  </si>
+  <si>
+    <t>Type</t>
+  </si>
+  <si>
+    <t>Component Source Type</t>
+  </si>
+  <si>
+    <t>Hash (SHA-1)</t>
+  </si>
+  <si>
+    <t>Hash (SHA-256)</t>
+  </si>
+  <si>
+    <t>PURL</t>
+  </si>
+  <si>
+    <t>Packaging</t>
+  </si>
+  <si>
+    <t>Path in Asset</t>
+  </si>
+  <si>
+    <t>log4j-api-2.14.0.jar</t>
+  </si>
+  <si>
+    <t>c</t>
+  </si>
+  <si>
+    <t>4876a0d414b3c2a01c10b6e96d70b62d</t>
+  </si>
+  <si>
+    <t>Apache Log4j</t>
+  </si>
+  <si>
+    <t>org.apache.logging.log4j</t>
+  </si>
+  <si>
+    <t>2.14.0</t>
+  </si>
+  <si>
+    <t>module</t>
+  </si>
+  <si>
+    <t>jar-module</t>
+  </si>
+  <si>
+    <t>23cdb2c6babad9b2b0dcf47c6a2c29d504e4c7a8</t>
+  </si>
+  <si>
+    <t>9791ac85aa3cdad633e512192766f84995eddf4db188cc42facec52a0dae15e8</t>
+  </si>
+  <si>
+    <t>pkg:maven/org.apache.logging.log4j/log4j-api@2.14.0?type=jar</t>
+  </si>
+  <si>
+    <t>jar</t>
+  </si>
+  <si>
+    <t>log4j-core-2.14.0.jar</t>
+  </si>
+  <si>
+    <t>862c00b2e854f9c0f1e8d8409d23d899</t>
+  </si>
+  <si>
+    <t>e257b0562453f73eabac1bc3181ba33e79d193ed</t>
+  </si>
+  <si>
+    <t>f04ee9c0ac417471d9127b5880b96c3147249f20674a8dbb88e9949d855382a8</t>
+  </si>
+  <si>
+    <t>pkg:maven/org.apache.logging.log4j/log4j-core@2.14.0?type=jar</t>
+  </si>
+  <si>
+    <t>spring-aop-5.3.14.jar</t>
+  </si>
+  <si>
+    <t>953a41d016a5bc9d9e8ace3d90d499c9</t>
+  </si>
+  <si>
+    <t>Spring Framework</t>
+  </si>
+  <si>
+    <t>org.springframework</t>
+  </si>
+  <si>
+    <t>5.3.14</t>
+  </si>
+  <si>
+    <t>f049146a55991e89c0f04b9624f1f69e1763d80f</t>
+  </si>
+  <si>
+    <t>1f6bb90bc78fa69506841c24c33f29790650e092dab96a35e56441f045ae216d</t>
+  </si>
+  <si>
+    <t>spring-beans-5.3.14.jar</t>
+  </si>
+  <si>
+    <t>04f9dc60a62319c97f140b8ebc98f797</t>
+  </si>
+  <si>
+    <t>24cc27af89edc1581a57bb15bc160d2353f40a0e</t>
+  </si>
+  <si>
+    <t>b354f54923139b8d86bc594452a6f53329da7b1e0c2a6402f9d9ca24837091ad</t>
+  </si>
+  <si>
+    <t>spring-context-5.3.14.jar</t>
+  </si>
+  <si>
+    <t>731eee1b78fa01375de10fd95b84455d</t>
+  </si>
+  <si>
+    <t>ce6042492f042131f602bdc83fcb412b142bdac5</t>
+  </si>
+  <si>
+    <t>25efd823c10f3afbe1b65efe97370def475d202dd91477f66eb5685e746e2819</t>
+  </si>
+  <si>
+    <t>spring-core-5.3.14.jar</t>
+  </si>
+  <si>
+    <t>b9d1f2454c4b7d94c058026d272dfc3c</t>
+  </si>
+  <si>
+    <t>d87ad19f9d8b9a3f1a143db5a2be34c61751aaa2</t>
+  </si>
+  <si>
+    <t>00ffcfb2671e0c8cab33f75939c97e04127fcfd2e0670032c59b6f48d791b772</t>
+  </si>
+  <si>
+    <t>spring-expression-5.3.14.jar</t>
+  </si>
+  <si>
+    <t>1d268dba90b89964d97254bae133a431</t>
+  </si>
+  <si>
+    <t>5cd4c568522b7084afac5d2ac6cb945b797b3f16</t>
+  </si>
+  <si>
+    <t>f196833d5bca28b12fbb4ae3265c0f0c4dc9fb4c726b3bfc4cabcc129cd21cf7</t>
+  </si>
+  <si>
+    <t>spring-jcl-5.3.14.jar</t>
+  </si>
+  <si>
+    <t>dd81ad7cd0aa5b6f0225d6a0341edd9a</t>
+  </si>
+  <si>
+    <t>ffcf745ed5ba32930771378316fd08e97986bec2</t>
+  </si>
+  <si>
+    <t>b522a60d1f37b8f8b3b6ab58617df850b55fee6d82011b879a62574e068946aa</t>
+  </si>
+  <si>
     <t>License</t>
   </si>
   <si>
@@ -122,12 +323,6 @@
   </si>
   <si>
     <t>Comment</t>
-  </si>
-  <si>
-    <t>Spring Framework</t>
-  </si>
-  <si>
-    <t>5.3.14</t>
   </si>
   <si>
     <t>Apache License 2.0, BSD 3-Clause License (copyright holder variant)</t>
@@ -147,201 +342,6 @@
 &lt;p&gt;The subcomponent &lt;b&gt;CGLIB 3.3&lt;/b&gt; is licensed under the terms of the Apache License 2.0.&lt;/p&gt;
 &lt;p&gt;The subcomponent &lt;b&gt;Objenesis 3.1&lt;/b&gt; is licensed under the terms of the Apache License 2.0.&lt;/p&gt;
 &lt;p&gt;Per the NOTICE file in the Objenesis ZIP distribution downloaded from http://objenesis.org/download.html and corresponding to section 4d of the Apache License, Version 2.0, in this case for Objenesis:&lt;lq&gt;Objenesis Copyright 2006-2019 Joe Walnes, Henri Tremblay, Leonardo Mesquita&lt;/lq&gt;&lt;/p&gt;</t>
-  </si>
-  <si>
-    <t>Assessment-Context</t>
-  </si>
-  <si>
-    <t>Asset-Id</t>
-  </si>
-  <si>
-    <t>Footer</t>
-  </si>
-  <si>
-    <t>Subtitle</t>
-  </si>
-  <si>
-    <t>Tenant</t>
-  </si>
-  <si>
-    <t>Title</t>
-  </si>
-  <si>
-    <t>vad-customization</t>
-  </si>
-  <si>
-    <t>local</t>
-  </si>
-  <si>
-    <t>sample-product-1</t>
-  </si>
-  <si>
-    <t>advise_enrich-inventory</t>
-  </si>
-  <si>
-    <t>metaeffekt</t>
-  </si>
-  <si>
-    <t>Vulnerability Assessment Dashboard</t>
-  </si>
-  <si>
-    <t>CID-8ddfbf9408625337e69608156e0a075016b427b672d796cd694450222f88ac23</t>
-  </si>
-  <si>
-    <t>Checksum</t>
-  </si>
-  <si>
-    <t>Group Id</t>
-  </si>
-  <si>
-    <t>Projects</t>
-  </si>
-  <si>
-    <t>Type</t>
-  </si>
-  <si>
-    <t>Component Source Type</t>
-  </si>
-  <si>
-    <t>Hash (SHA-1)</t>
-  </si>
-  <si>
-    <t>Hash (SHA-256)</t>
-  </si>
-  <si>
-    <t>PURL</t>
-  </si>
-  <si>
-    <t>Packaging</t>
-  </si>
-  <si>
-    <t>Path in Asset</t>
-  </si>
-  <si>
-    <t>log4j-api-2.14.0.jar</t>
-  </si>
-  <si>
-    <t>c</t>
-  </si>
-  <si>
-    <t>4876a0d414b3c2a01c10b6e96d70b62d</t>
-  </si>
-  <si>
-    <t>Apache Log4j</t>
-  </si>
-  <si>
-    <t>org.apache.logging.log4j</t>
-  </si>
-  <si>
-    <t>2.14.0</t>
-  </si>
-  <si>
-    <t>module</t>
-  </si>
-  <si>
-    <t>jar-module</t>
-  </si>
-  <si>
-    <t>23cdb2c6babad9b2b0dcf47c6a2c29d504e4c7a8</t>
-  </si>
-  <si>
-    <t>9791ac85aa3cdad633e512192766f84995eddf4db188cc42facec52a0dae15e8</t>
-  </si>
-  <si>
-    <t>pkg:maven/org.apache.logging.log4j/log4j-api@2.14.0?type=jar</t>
-  </si>
-  <si>
-    <t>jar</t>
-  </si>
-  <si>
-    <t>log4j-core-2.14.0.jar</t>
-  </si>
-  <si>
-    <t>862c00b2e854f9c0f1e8d8409d23d899</t>
-  </si>
-  <si>
-    <t>e257b0562453f73eabac1bc3181ba33e79d193ed</t>
-  </si>
-  <si>
-    <t>f04ee9c0ac417471d9127b5880b96c3147249f20674a8dbb88e9949d855382a8</t>
-  </si>
-  <si>
-    <t>pkg:maven/org.apache.logging.log4j/log4j-core@2.14.0?type=jar</t>
-  </si>
-  <si>
-    <t>spring-aop-5.3.14.jar</t>
-  </si>
-  <si>
-    <t>953a41d016a5bc9d9e8ace3d90d499c9</t>
-  </si>
-  <si>
-    <t>org.springframework</t>
-  </si>
-  <si>
-    <t>f049146a55991e89c0f04b9624f1f69e1763d80f</t>
-  </si>
-  <si>
-    <t>1f6bb90bc78fa69506841c24c33f29790650e092dab96a35e56441f045ae216d</t>
-  </si>
-  <si>
-    <t>spring-beans-5.3.14.jar</t>
-  </si>
-  <si>
-    <t>04f9dc60a62319c97f140b8ebc98f797</t>
-  </si>
-  <si>
-    <t>24cc27af89edc1581a57bb15bc160d2353f40a0e</t>
-  </si>
-  <si>
-    <t>b354f54923139b8d86bc594452a6f53329da7b1e0c2a6402f9d9ca24837091ad</t>
-  </si>
-  <si>
-    <t>spring-context-5.3.14.jar</t>
-  </si>
-  <si>
-    <t>731eee1b78fa01375de10fd95b84455d</t>
-  </si>
-  <si>
-    <t>ce6042492f042131f602bdc83fcb412b142bdac5</t>
-  </si>
-  <si>
-    <t>25efd823c10f3afbe1b65efe97370def475d202dd91477f66eb5685e746e2819</t>
-  </si>
-  <si>
-    <t>spring-core-5.3.14.jar</t>
-  </si>
-  <si>
-    <t>b9d1f2454c4b7d94c058026d272dfc3c</t>
-  </si>
-  <si>
-    <t>d87ad19f9d8b9a3f1a143db5a2be34c61751aaa2</t>
-  </si>
-  <si>
-    <t>00ffcfb2671e0c8cab33f75939c97e04127fcfd2e0670032c59b6f48d791b772</t>
-  </si>
-  <si>
-    <t>spring-expression-5.3.14.jar</t>
-  </si>
-  <si>
-    <t>1d268dba90b89964d97254bae133a431</t>
-  </si>
-  <si>
-    <t>5cd4c568522b7084afac5d2ac6cb945b797b3f16</t>
-  </si>
-  <si>
-    <t>f196833d5bca28b12fbb4ae3265c0f0c4dc9fb4c726b3bfc4cabcc129cd21cf7</t>
-  </si>
-  <si>
-    <t>spring-jcl-5.3.14.jar</t>
-  </si>
-  <si>
-    <t>dd81ad7cd0aa5b6f0225d6a0341edd9a</t>
-  </si>
-  <si>
-    <t>ffcf745ed5ba32930771378316fd08e97986bec2</t>
-  </si>
-  <si>
-    <t>b522a60d1f37b8f8b3b6ab58617df850b55fee6d82011b879a62574e068946aa</t>
   </si>
   <si>
     <t>Asset Id</t>
@@ -751,377 +751,377 @@
         <v>1</v>
       </c>
       <c r="B1" s="4" t="s">
+        <v>38</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="I1" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="J1" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="K1" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="L1" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="M1" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="N1" s="1" t="s">
         <v>50</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>51</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>26</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>52</v>
-      </c>
-      <c r="F1" s="1" t="s">
-        <v>27</v>
-      </c>
-      <c r="G1" s="1" t="s">
-        <v>53</v>
-      </c>
-      <c r="H1" s="1" t="s">
-        <v>54</v>
-      </c>
-      <c r="I1" s="1" t="s">
-        <v>55</v>
-      </c>
-      <c r="J1" s="1" t="s">
-        <v>56</v>
-      </c>
-      <c r="K1" s="1" t="s">
-        <v>57</v>
-      </c>
-      <c r="L1" s="1" t="s">
-        <v>58</v>
-      </c>
-      <c r="M1" s="1" t="s">
-        <v>59</v>
-      </c>
-      <c r="N1" s="1" t="s">
-        <v>60</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="s">
+        <v>51</v>
+      </c>
+      <c r="B2" s="9" t="s">
+        <v>52</v>
+      </c>
+      <c r="C2" t="s">
+        <v>53</v>
+      </c>
+      <c r="D2" t="s">
+        <v>54</v>
+      </c>
+      <c r="E2" t="s">
+        <v>55</v>
+      </c>
+      <c r="F2" t="s">
+        <v>56</v>
+      </c>
+      <c r="G2" t="s">
+        <v>51</v>
+      </c>
+      <c r="H2" t="s">
+        <v>57</v>
+      </c>
+      <c r="I2" t="s">
+        <v>58</v>
+      </c>
+      <c r="J2" t="s">
+        <v>59</v>
+      </c>
+      <c r="K2" t="s">
+        <v>60</v>
+      </c>
+      <c r="L2" t="s">
         <v>61</v>
       </c>
-      <c r="B2" s="9" t="s">
+      <c r="M2" t="s">
         <v>62</v>
       </c>
-      <c r="C2" t="s">
-        <v>63</v>
-      </c>
-      <c r="D2" t="s">
-        <v>64</v>
-      </c>
-      <c r="E2" t="s">
-        <v>65</v>
-      </c>
-      <c r="F2" t="s">
-        <v>66</v>
-      </c>
-      <c r="G2" t="s">
-        <v>61</v>
-      </c>
-      <c r="H2" t="s">
-        <v>67</v>
-      </c>
-      <c r="I2" t="s">
-        <v>68</v>
-      </c>
-      <c r="J2" t="s">
-        <v>69</v>
-      </c>
-      <c r="K2" t="s">
-        <v>70</v>
-      </c>
-      <c r="L2" t="s">
-        <v>71</v>
-      </c>
-      <c r="M2" t="s">
-        <v>72</v>
-      </c>
       <c r="N2" t="s">
-        <v>61</v>
+        <v>51</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>73</v>
+        <v>63</v>
       </c>
       <c r="B3" s="9" t="s">
+        <v>52</v>
+      </c>
+      <c r="C3" t="s">
+        <v>64</v>
+      </c>
+      <c r="D3" t="s">
+        <v>54</v>
+      </c>
+      <c r="E3" t="s">
+        <v>55</v>
+      </c>
+      <c r="F3" t="s">
+        <v>56</v>
+      </c>
+      <c r="G3" t="s">
+        <v>63</v>
+      </c>
+      <c r="H3" t="s">
+        <v>57</v>
+      </c>
+      <c r="I3" t="s">
+        <v>58</v>
+      </c>
+      <c r="J3" t="s">
+        <v>65</v>
+      </c>
+      <c r="K3" t="s">
+        <v>66</v>
+      </c>
+      <c r="L3" t="s">
+        <v>67</v>
+      </c>
+      <c r="M3" t="s">
         <v>62</v>
       </c>
-      <c r="C3" t="s">
-        <v>74</v>
-      </c>
-      <c r="D3" t="s">
-        <v>64</v>
-      </c>
-      <c r="E3" t="s">
-        <v>65</v>
-      </c>
-      <c r="F3" t="s">
-        <v>66</v>
-      </c>
-      <c r="G3" t="s">
-        <v>73</v>
-      </c>
-      <c r="H3" t="s">
-        <v>67</v>
-      </c>
-      <c r="I3" t="s">
-        <v>68</v>
-      </c>
-      <c r="J3" t="s">
-        <v>75</v>
-      </c>
-      <c r="K3" t="s">
-        <v>76</v>
-      </c>
-      <c r="L3" t="s">
-        <v>77</v>
-      </c>
-      <c r="M3" t="s">
-        <v>72</v>
-      </c>
       <c r="N3" t="s">
-        <v>73</v>
+        <v>63</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>78</v>
+        <v>68</v>
       </c>
       <c r="B4" s="9" t="s">
+        <v>52</v>
+      </c>
+      <c r="C4" t="s">
+        <v>69</v>
+      </c>
+      <c r="D4" t="s">
+        <v>70</v>
+      </c>
+      <c r="E4" t="s">
+        <v>71</v>
+      </c>
+      <c r="F4" t="s">
+        <v>72</v>
+      </c>
+      <c r="G4" t="s">
+        <v>68</v>
+      </c>
+      <c r="H4" t="s">
+        <v>57</v>
+      </c>
+      <c r="I4" t="s">
+        <v>58</v>
+      </c>
+      <c r="J4" t="s">
+        <v>73</v>
+      </c>
+      <c r="K4" t="s">
+        <v>74</v>
+      </c>
+      <c r="M4" t="s">
         <v>62</v>
       </c>
-      <c r="C4" t="s">
-        <v>79</v>
-      </c>
-      <c r="D4" t="s">
-        <v>33</v>
-      </c>
-      <c r="E4" t="s">
-        <v>80</v>
-      </c>
-      <c r="F4" t="s">
-        <v>34</v>
-      </c>
-      <c r="G4" t="s">
-        <v>78</v>
-      </c>
-      <c r="H4" t="s">
-        <v>67</v>
-      </c>
-      <c r="I4" t="s">
+      <c r="N4" t="s">
         <v>68</v>
-      </c>
-      <c r="J4" t="s">
-        <v>81</v>
-      </c>
-      <c r="K4" t="s">
-        <v>82</v>
-      </c>
-      <c r="M4" t="s">
-        <v>72</v>
-      </c>
-      <c r="N4" t="s">
-        <v>78</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>83</v>
+        <v>75</v>
       </c>
       <c r="B5" s="9" t="s">
+        <v>52</v>
+      </c>
+      <c r="C5" t="s">
+        <v>76</v>
+      </c>
+      <c r="D5" t="s">
+        <v>70</v>
+      </c>
+      <c r="E5" t="s">
+        <v>71</v>
+      </c>
+      <c r="F5" t="s">
+        <v>72</v>
+      </c>
+      <c r="G5" t="s">
+        <v>75</v>
+      </c>
+      <c r="H5" t="s">
+        <v>57</v>
+      </c>
+      <c r="I5" t="s">
+        <v>58</v>
+      </c>
+      <c r="J5" t="s">
+        <v>77</v>
+      </c>
+      <c r="K5" t="s">
+        <v>78</v>
+      </c>
+      <c r="M5" t="s">
         <v>62</v>
       </c>
-      <c r="C5" t="s">
-        <v>84</v>
-      </c>
-      <c r="D5" t="s">
-        <v>33</v>
-      </c>
-      <c r="E5" t="s">
-        <v>80</v>
-      </c>
-      <c r="F5" t="s">
-        <v>34</v>
-      </c>
-      <c r="G5" t="s">
-        <v>83</v>
-      </c>
-      <c r="H5" t="s">
-        <v>67</v>
-      </c>
-      <c r="I5" t="s">
-        <v>68</v>
-      </c>
-      <c r="J5" t="s">
-        <v>85</v>
-      </c>
-      <c r="K5" t="s">
-        <v>86</v>
-      </c>
-      <c r="M5" t="s">
-        <v>72</v>
-      </c>
       <c r="N5" t="s">
-        <v>83</v>
+        <v>75</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="s">
-        <v>87</v>
+        <v>79</v>
       </c>
       <c r="B6" s="9" t="s">
+        <v>52</v>
+      </c>
+      <c r="C6" t="s">
+        <v>80</v>
+      </c>
+      <c r="D6" t="s">
+        <v>70</v>
+      </c>
+      <c r="E6" t="s">
+        <v>71</v>
+      </c>
+      <c r="F6" t="s">
+        <v>72</v>
+      </c>
+      <c r="G6" t="s">
+        <v>79</v>
+      </c>
+      <c r="H6" t="s">
+        <v>57</v>
+      </c>
+      <c r="I6" t="s">
+        <v>58</v>
+      </c>
+      <c r="J6" t="s">
+        <v>81</v>
+      </c>
+      <c r="K6" t="s">
+        <v>82</v>
+      </c>
+      <c r="M6" t="s">
         <v>62</v>
       </c>
-      <c r="C6" t="s">
-        <v>88</v>
-      </c>
-      <c r="D6" t="s">
-        <v>33</v>
-      </c>
-      <c r="E6" t="s">
-        <v>80</v>
-      </c>
-      <c r="F6" t="s">
-        <v>34</v>
-      </c>
-      <c r="G6" t="s">
-        <v>87</v>
-      </c>
-      <c r="H6" t="s">
-        <v>67</v>
-      </c>
-      <c r="I6" t="s">
-        <v>68</v>
-      </c>
-      <c r="J6" t="s">
-        <v>89</v>
-      </c>
-      <c r="K6" t="s">
-        <v>90</v>
-      </c>
-      <c r="M6" t="s">
-        <v>72</v>
-      </c>
       <c r="N6" t="s">
-        <v>87</v>
+        <v>79</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="s">
-        <v>91</v>
+        <v>83</v>
       </c>
       <c r="B7" s="9" t="s">
+        <v>52</v>
+      </c>
+      <c r="C7" t="s">
+        <v>84</v>
+      </c>
+      <c r="D7" t="s">
+        <v>70</v>
+      </c>
+      <c r="E7" t="s">
+        <v>71</v>
+      </c>
+      <c r="F7" t="s">
+        <v>72</v>
+      </c>
+      <c r="G7" t="s">
+        <v>83</v>
+      </c>
+      <c r="H7" t="s">
+        <v>57</v>
+      </c>
+      <c r="I7" t="s">
+        <v>58</v>
+      </c>
+      <c r="J7" t="s">
+        <v>85</v>
+      </c>
+      <c r="K7" t="s">
+        <v>86</v>
+      </c>
+      <c r="M7" t="s">
         <v>62</v>
       </c>
-      <c r="C7" t="s">
-        <v>92</v>
-      </c>
-      <c r="D7" t="s">
-        <v>33</v>
-      </c>
-      <c r="E7" t="s">
-        <v>80</v>
-      </c>
-      <c r="F7" t="s">
-        <v>34</v>
-      </c>
-      <c r="G7" t="s">
-        <v>91</v>
-      </c>
-      <c r="H7" t="s">
-        <v>67</v>
-      </c>
-      <c r="I7" t="s">
-        <v>68</v>
-      </c>
-      <c r="J7" t="s">
-        <v>93</v>
-      </c>
-      <c r="K7" t="s">
-        <v>94</v>
-      </c>
-      <c r="M7" t="s">
-        <v>72</v>
-      </c>
       <c r="N7" t="s">
-        <v>91</v>
+        <v>83</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="s">
-        <v>95</v>
+        <v>87</v>
       </c>
       <c r="B8" s="9" t="s">
+        <v>52</v>
+      </c>
+      <c r="C8" t="s">
+        <v>88</v>
+      </c>
+      <c r="D8" t="s">
+        <v>70</v>
+      </c>
+      <c r="E8" t="s">
+        <v>71</v>
+      </c>
+      <c r="F8" t="s">
+        <v>72</v>
+      </c>
+      <c r="G8" t="s">
+        <v>87</v>
+      </c>
+      <c r="H8" t="s">
+        <v>57</v>
+      </c>
+      <c r="I8" t="s">
+        <v>58</v>
+      </c>
+      <c r="J8" t="s">
+        <v>89</v>
+      </c>
+      <c r="K8" t="s">
+        <v>90</v>
+      </c>
+      <c r="M8" t="s">
         <v>62</v>
       </c>
-      <c r="C8" t="s">
-        <v>96</v>
-      </c>
-      <c r="D8" t="s">
-        <v>33</v>
-      </c>
-      <c r="E8" t="s">
-        <v>80</v>
-      </c>
-      <c r="F8" t="s">
-        <v>34</v>
-      </c>
-      <c r="G8" t="s">
-        <v>95</v>
-      </c>
-      <c r="H8" t="s">
-        <v>67</v>
-      </c>
-      <c r="I8" t="s">
-        <v>68</v>
-      </c>
-      <c r="J8" t="s">
-        <v>97</v>
-      </c>
-      <c r="K8" t="s">
-        <v>98</v>
-      </c>
-      <c r="M8" t="s">
-        <v>72</v>
-      </c>
       <c r="N8" t="s">
-        <v>95</v>
+        <v>87</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="s">
-        <v>99</v>
+        <v>91</v>
       </c>
       <c r="B9" s="9" t="s">
+        <v>52</v>
+      </c>
+      <c r="C9" t="s">
+        <v>92</v>
+      </c>
+      <c r="D9" t="s">
+        <v>70</v>
+      </c>
+      <c r="E9" t="s">
+        <v>71</v>
+      </c>
+      <c r="F9" t="s">
+        <v>72</v>
+      </c>
+      <c r="G9" t="s">
+        <v>91</v>
+      </c>
+      <c r="H9" t="s">
+        <v>57</v>
+      </c>
+      <c r="I9" t="s">
+        <v>58</v>
+      </c>
+      <c r="J9" t="s">
+        <v>93</v>
+      </c>
+      <c r="K9" t="s">
+        <v>94</v>
+      </c>
+      <c r="M9" t="s">
         <v>62</v>
       </c>
-      <c r="C9" t="s">
-        <v>100</v>
-      </c>
-      <c r="D9" t="s">
-        <v>33</v>
-      </c>
-      <c r="E9" t="s">
-        <v>80</v>
-      </c>
-      <c r="F9" t="s">
-        <v>34</v>
-      </c>
-      <c r="G9" t="s">
-        <v>99</v>
-      </c>
-      <c r="H9" t="s">
-        <v>67</v>
-      </c>
-      <c r="I9" t="s">
-        <v>68</v>
-      </c>
-      <c r="J9" t="s">
-        <v>101</v>
-      </c>
-      <c r="K9" t="s">
-        <v>102</v>
-      </c>
-      <c r="M9" t="s">
-        <v>72</v>
-      </c>
       <c r="N9" t="s">
-        <v>99</v>
+        <v>91</v>
       </c>
     </row>
   </sheetData>
@@ -1172,10 +1172,10 @@
         <v>105</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>51</v>
+        <v>39</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>32</v>
+        <v>99</v>
       </c>
       <c r="F1" s="1" t="s">
         <v>106</v>
@@ -1208,13 +1208,13 @@
         <v>115</v>
       </c>
       <c r="P1" s="1" t="s">
-        <v>54</v>
+        <v>44</v>
       </c>
       <c r="Q1" s="1" t="s">
         <v>116</v>
       </c>
       <c r="R1" s="1" t="s">
-        <v>27</v>
+        <v>42</v>
       </c>
       <c r="S1" s="3" t="s">
         <v>117</v>
@@ -1291,7 +1291,7 @@
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>50</v>
+        <v>38</v>
       </c>
       <c r="B2" t="s">
         <v>141</v>
@@ -1430,42 +1430,42 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="s">
-        <v>26</v>
+        <v>40</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>27</v>
+        <v>42</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>28</v>
+        <v>95</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>29</v>
+        <v>96</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>30</v>
+        <v>97</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>31</v>
+        <v>98</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>32</v>
+        <v>99</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>33</v>
+        <v>70</v>
       </c>
       <c r="B2" t="s">
-        <v>34</v>
+        <v>72</v>
       </c>
       <c r="C2" t="s">
-        <v>35</v>
+        <v>100</v>
       </c>
       <c r="D2" t="s">
-        <v>36</v>
+        <v>101</v>
       </c>
       <c r="F2" t="s">
-        <v>37</v>
+        <v>102</v>
       </c>
     </row>
   </sheetData>
@@ -1642,45 +1642,45 @@
         <v>1</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>38</v>
+        <v>26</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>39</v>
+        <v>27</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>40</v>
+        <v>28</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>41</v>
+        <v>29</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>42</v>
+        <v>30</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>43</v>
+        <v>31</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>44</v>
+        <v>32</v>
       </c>
       <c r="B2" t="s">
-        <v>45</v>
+        <v>33</v>
       </c>
       <c r="C2" t="s">
-        <v>46</v>
+        <v>34</v>
       </c>
       <c r="D2" t="s">
-        <v>47</v>
+        <v>35</v>
       </c>
       <c r="E2" t="s">
-        <v>47</v>
+        <v>35</v>
       </c>
       <c r="F2" t="s">
-        <v>48</v>
+        <v>36</v>
       </c>
       <c r="G2" t="s">
-        <v>49</v>
+        <v>37</v>
       </c>
     </row>
   </sheetData>

</xml_diff>